<commit_message>
Auto scrape + SQL (from Excel) 2025-11-24 17:17:15
</commit_message>
<xml_diff>
--- a/nhatot_phongtro_danang_all.xlsx
+++ b/nhatot_phongtro_danang_all.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J153"/>
+  <dimension ref="A1:J152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -483,27 +483,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Nhà nguyên căn, dt 100m2, 234/10 Đỗ Bá</t>
+          <t>Phòng trọ ngay cầu rồng hướng ra biển, giá 2,9tr</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>7 triệu/tháng</t>
+          <t>2,9 triệu/tháng</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>100 m²</t>
+          <t>15 m²</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -520,38 +520,38 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129258007.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129279640.htm</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Cho thuê nguyên tầng 3, diện tích 100m2</t>
+          <t>Cho thuê phòng trọ</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>5 triệu/tháng</t>
+          <t>2 triệu/tháng</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>100 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -560,28 +560,28 @@
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129257747.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129278299.htm</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>phòng trong nhà mặt tiền hoàng diệu</t>
+          <t>cho thuê giường dorm</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>3,3 triệu/tháng</t>
+          <t>1,4 triệu/tháng</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>38 m²</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -591,14 +591,14 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F4" t="n">
         <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4" t="n">
         <v>1</v>
@@ -608,41 +608,41 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128458947.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/126893939.htm</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Cho Thuê Trọ Kiệt Chế Lan Viên</t>
+          <t>MỜI BẠN VỀ NHÀ</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1,5 triệu/tháng</t>
+          <t>7 triệu/tháng</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>10 m²</t>
+          <t>68.8 m²</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
@@ -652,73 +652,73 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129256726.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128979633.htm</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CHO THUÊ PHÒNG TRỌ SẠCH SẼ MÁT MẺ TRONG NHÀ 4 TẦNG KHU VỰC THANH KHÊ</t>
+          <t>Phòng trọ nhỏ giá cả hợp lí đường Nguyễn Công Trứ gần cầu Rồng</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1,8 triệu/tháng</t>
+          <t>2,9 triệu/tháng</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>15 m²</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129251296.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/127178277.htm</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Phòng trọ nội thất cơ bản</t>
+          <t>CHO THUÊ PHÒNG TRỌ SẠCH SẼ MÁT MẺ TRONG NHÀ 4 TẦNG KHU VỰC THANH KHÊ</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2,5 triệu/tháng</t>
+          <t>1,8 triệu/tháng</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>18 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -736,28 +736,28 @@
         <v>1</v>
       </c>
       <c r="I7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129239038.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129251296.htm</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Nhà trọ sang chảnh</t>
+          <t>Cho thuê phòng đầy đủ tiện nghi,khu ngã ba huế,bến xe</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2,7 triệu/tháng</t>
+          <t>1,8 triệu/tháng</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17 m²</t>
+          <t>15 m²</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -767,14 +767,14 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F8" t="n">
         <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
@@ -784,19 +784,19 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/127668535.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128606799.htm</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Nhà trọ Văn Minh có 1 phòng trống</t>
+          <t>TRỌ GÁC LỬNG 25M2 CHỈ 1.8TR TRONG MẶT TIỀN KIỀU PHỤNG RIÊNG CHỦ</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2,2 triệu/tháng</t>
+          <t>1,8 triệu/tháng</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -806,12 +806,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -828,29 +828,29 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129229044.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129266347.htm</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Cho thuê phòng đầy đủ tiện nghi,khu ngã ba huế,bến xe</t>
+          <t>phòng trong nhà mặt tiền hoàng diệu</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>1,8 triệu/tháng</t>
+          <t>3,3 triệu/tháng</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>15 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -862,39 +862,39 @@
         <v>1</v>
       </c>
       <c r="G10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128606799.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128458947.htm</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>cho thuê phòng trọ phường Hải Châu</t>
+          <t>PHÒNG TRỌ GẦN CẦU VƯỢT NGÃ BA HUẾ ĐÀ NẴNG</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>3,5 triệu/tháng</t>
+          <t>1,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>32 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -903,37 +903,37 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129246849.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129265301.htm</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ (Chung chủ)</t>
+          <t>Căn hộ mini full nội thất Sơn Trà</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>3 triệu/tháng</t>
+          <t>3,8 triệu/tháng</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -947,86 +947,86 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129246276.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128837798.htm</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ tại 508 Lê Văn Hiến, Ngũ Hành Sơn, TP. Đà Nẵng</t>
+          <t>Phòng trọ full nội thất đối diện siêu thị Go</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1,5 triệu/tháng</t>
+          <t>4,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129243560.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129260352.htm</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ rộng rãi, an ninh, gần các trường học</t>
+          <t>Nhà nguyên căn, dt 100m2, 234/10 Đỗ Bá</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2,4 triệu/tháng</t>
+          <t>7 triệu/tháng</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>100 m²</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1044,33 +1044,33 @@
         <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129237617.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129258007.htm</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Phòng ban công full nội thất new 100% khu FPT - Ngũ Hành Sơn</t>
+          <t>Cho thuê nguyên tầng 3, diện tích 100m2</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>4 triệu/tháng</t>
+          <t>5 triệu/tháng</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>40 m²</t>
+          <t>100 m²</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1085,41 +1085,41 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I15" t="n">
         <v>1</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128629777.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129257747.htm</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Phòng Full Nội Thất Khu FPT - Ngũ Hành Sơn</t>
+          <t>Phòng trọ nội thất cơ bản</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>3,9 triệu/tháng</t>
+          <t>2,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>40 m²</t>
+          <t>18 m²</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -1129,109 +1129,109 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128025078.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129239038.htm</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>phòng cho thuê trọ</t>
+          <t>Nhà trọ sang chảnh</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>3,6 triệu/tháng</t>
+          <t>2,7 triệu/tháng</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>28 m²</t>
+          <t>17 m²</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F17" t="n">
         <v>1</v>
       </c>
       <c r="G17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129192954.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/127668535.htm</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Cho thuê phòng full option. 129  Nguyễn Khánh Toàn Trung Tâm Đà Nẵng</t>
+          <t>Nhà trọ Văn Minh có 1 phòng trống</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>4,3 triệu/tháng</t>
+          <t>2,2 triệu/tháng</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I18" t="n">
         <v>0</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128845940.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129229044.htm</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Cho Thuê trọ phòng khách sạn</t>
+          <t>cho thuê phòng trọ phường Hải Châu</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1241,41 +1241,41 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>32 m²</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F19" t="n">
         <v>1</v>
       </c>
       <c r="G19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/127808442.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129246849.htm</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Phòng trọ 17m2 Đường Lương Thế Vinh Quận Sơn Trà</t>
+          <t>Cho thuê phòng trọ (Chung chủ)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>17 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F20" t="n">
@@ -1312,34 +1312,34 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129201071.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129246276.htm</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>căn hộ tại 240/6 lê duẩn</t>
+          <t>Cho thuê phòng trọ tại 508 Lê Văn Hiến, Ngũ Hành Sơn, TP. Đà Nẵng</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>3 triệu/tháng</t>
+          <t>1,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>18 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F21" t="n">
@@ -1356,24 +1356,24 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129220491.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129243560.htm</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Phòng trọ 35mv đg Ng Trung Trực - cách Sông Hàn 1km- gần tr Greenwich</t>
+          <t>phòng Cho Thuê  tầng  2 - cửa sổ ban công thoáng mát</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>3,5 triệu/tháng</t>
+          <t>2,8 triệu/tháng</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>35 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F22" t="n">
@@ -1396,33 +1396,33 @@
         <v>0</v>
       </c>
       <c r="I22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129229623.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/127699774.htm</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ 1tr5</t>
+          <t>Cho thuê phòng trọ rộng rãi, an ninh, gần các trường học</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1,5 triệu/tháng</t>
+          <t>2,4 triệu/tháng</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1444,29 +1444,29 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129225686.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129237617.htm</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>cho thuê căn hộ mini</t>
+          <t>Phòng ban công full nội thất new 100% khu FPT - Ngũ Hành Sơn</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>3 triệu/tháng</t>
+          <t>4 triệu/tháng</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>40 m²</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1484,174 +1484,174 @@
         <v>1</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128670490.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128629777.htm</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ đường Châu Văn Liêm, gần Vũ Trường Phương Đông</t>
+          <t>Phòng Full Nội Thất Khu FPT - Ngũ Hành Sơn</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>3,7 triệu/tháng</t>
+          <t>3,9 triệu/tháng</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>32 m²</t>
+          <t>40 m²</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Nội thất cao cấp</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F25" t="n">
         <v>1</v>
       </c>
       <c r="G25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128605782.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128025078.htm</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Phòng trọ giá tốt</t>
+          <t>phòng cho thuê trọ</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>950000 đ/tháng</t>
+          <t>3,6 triệu/tháng</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>12 m²</t>
+          <t>28 m²</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I26" t="n">
         <v>0</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129011618.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129192954.htm</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Trống 1 căn , full nội thất , phòng ngủ tách biệt</t>
+          <t>Cho thuê phòng full option. 129  Nguyễn Khánh Toàn Trung Tâm Đà Nẵng</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>4,1 triệu/tháng</t>
+          <t>4,3 triệu/tháng</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>40 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I27" t="n">
         <v>0</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129218959.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128845940.htm</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Cho thuê phòng mặt tiền 68/20 Nguyễn mộng tuân ngay bến xe</t>
+          <t>Cho Thuê trọ phòng khách sạn</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>4 triệu/tháng</t>
+          <t>3,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G28" t="n">
         <v>0</v>
@@ -1664,24 +1664,24 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129217669.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/127808442.htm</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Phòng trọ cho người độc thân tại sơn trà</t>
+          <t>Phòng trọ 17m2 Đường Lương Thế Vinh Quận Sơn Trà</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>1,7 triệu/tháng</t>
+          <t>3 triệu/tháng</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>400 m²</t>
+          <t>17 m²</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1691,7 +1691,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F29" t="n">
@@ -1708,29 +1708,29 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/125998127.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129201071.htm</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>phòng trọ gần cầu hoà xuân</t>
+          <t>căn hộ tại 240/6 lê duẩn</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>6 triệu/tháng</t>
+          <t>3 triệu/tháng</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>40 m²</t>
+          <t>18 m²</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1739,7 +1739,7 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G30" t="n">
         <v>0</v>
@@ -1752,29 +1752,29 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129199929.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129220491.htm</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>phòng trọ cao cấp</t>
+          <t>Phòng trọ 35mv đg Ng Trung Trực - cách Sông Hàn 1km- gần tr Greenwich</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>3 triệu/tháng</t>
+          <t>3,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>27 m²</t>
+          <t>35 m²</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1786,44 +1786,44 @@
         <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I31" t="n">
         <v>0</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/127030626.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129229623.htm</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Hoà Phú 27 Hoà Minh Liên Chiểu gần Mega market mới.</t>
+          <t>Cho thuê phòng trọ 1tr5</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>4,5 triệu/tháng</t>
+          <t>1,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>40 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F32" t="n">
@@ -1836,77 +1836,77 @@
         <v>0</v>
       </c>
       <c r="I32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129183180.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129225686.htm</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ riêng 68/20 Nguyễn mộng tuân</t>
+          <t>Cho thuê phòng trọ đường Châu Văn Liêm, gần Vũ Trường Phương Đông</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>4 triệu/tháng</t>
+          <t>3,7 triệu/tháng</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>32 m²</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất cao cấp</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128830619.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128605782.htm</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Phòng trọ 30m2 Hoà Xuân, an ninh, không chung chủ</t>
+          <t>Trống 1 căn , full nội thất , phòng ngủ tách biệt</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2,5 triệu/tháng</t>
+          <t>4,1 triệu/tháng</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>28 m²</t>
+          <t>40 m²</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1915,7 +1915,7 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G34" t="n">
         <v>0</v>
@@ -1928,14 +1928,14 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129184894.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129218959.htm</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>✨ Căn hộ mới 100% đi vào hoạt động</t>
+          <t>Cho thuê phòng mặt tiền 68/20 Nguyễn mộng tuân ngay bến xe</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1945,61 +1945,61 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129198937.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129217669.htm</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Phòng trọ tttp đường Hoàng Diệu sạch sẽ thoáng mát giờ giấc tự do</t>
+          <t>Phòng trọ cho người độc thân tại sơn trà</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>1,8 triệu/tháng</t>
+          <t>1,7 triệu/tháng</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>15 m²</t>
+          <t>400 m²</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F36" t="n">
@@ -2009,36 +2009,36 @@
         <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I36" t="n">
         <v>0</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129182091.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/125998127.htm</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ full nội thất</t>
+          <t>phòng trọ gần cầu hoà xuân</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>4,5 triệu/tháng</t>
+          <t>6 triệu/tháng</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>35 m²</t>
+          <t>40 m²</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2047,7 +2047,7 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G37" t="n">
         <v>0</v>
@@ -2060,24 +2060,24 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128820066.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129199929.htm</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CHO THUE PHONG TRO KCN HOA CAM CAM LE DA NANG</t>
+          <t>phòng trọ cao cấp</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>700000 đ/tháng</t>
+          <t>3 triệu/tháng</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>14 m²</t>
+          <t>27 m²</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2094,24 +2094,24 @@
         <v>0</v>
       </c>
       <c r="G38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I38" t="n">
         <v>0</v>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129009631.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/127030626.htm</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ gia đình</t>
+          <t>Hoà Phú 27 Hoà Minh Liên Chiểu gần Mega market mới.</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2121,46 +2121,46 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>60 m²</t>
+          <t>40 m²</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F39" t="n">
         <v>0</v>
       </c>
       <c r="G39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H39" t="n">
         <v>0</v>
       </c>
       <c r="I39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128786730.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129183180.htm</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>phòng 2 giường riêng .khách sạn sang trọng,ở ghép 2 người nam</t>
+          <t>Cho thuê phòng trọ riêng 68/20 Nguyễn mộng tuân</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>1,75 triệu/tháng</t>
+          <t>4 triệu/tháng</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2170,19 +2170,19 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Nội thất cao cấp</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F40" t="n">
         <v>0</v>
       </c>
       <c r="G40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H40" t="n">
         <v>0</v>
@@ -2192,38 +2192,38 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129197063.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128830619.htm</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Cho Thuê Phòng Thoáng Mát</t>
+          <t>Phòng trọ 30m2 Hoà Xuân, an ninh, không chung chủ</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>3,9 triệu/tháng</t>
+          <t>2,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>37 m²</t>
+          <t>28 m²</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G41" t="n">
         <v>0</v>
@@ -2236,73 +2236,73 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129191886.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129184894.htm</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ</t>
+          <t>✨ Căn hộ mới 100% đi vào hoạt động</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2,2 triệu/tháng</t>
+          <t>4 triệu/tháng</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>18 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129166725.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129198937.htm</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>💥💥💥💥💥Còn trống 1 phòng ***</t>
+          <t>Cho thuê phòng trọ full nội thất</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>3,5 triệu/tháng</t>
+          <t>4,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>28 m²</t>
+          <t>35 m²</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2317,36 +2317,36 @@
         <v>0</v>
       </c>
       <c r="H43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128498042.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128820066.htm</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Phòng trọ mới xây ngay trung tâm thành phố</t>
+          <t>CHO THUE PHONG TRO KCN HOA CAM CAM LE DA NANG</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>3 triệu/tháng</t>
+          <t>700000 đ/tháng</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16 m²</t>
+          <t>14 m²</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2361,92 +2361,92 @@
         <v>0</v>
       </c>
       <c r="H44" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I44" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129187653.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129009631.htm</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CHO THUÊ CĂN HỘ MỚI XÂY 100% - SỐ 17 CỒN DẦU 19 - HÒA XUÂN - CẨM LỆ</t>
+          <t>Cho thuê phòng trọ gia đình</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>4,8 triệu/tháng</t>
+          <t>4,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>60 m²</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H45" t="n">
         <v>0</v>
       </c>
       <c r="I45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128248490.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128786730.htm</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Cho thuê phòng đủ nội thất gần Đại học FPT, giá sinh viên</t>
+          <t>phòng 2 giường riêng .khách sạn sang trọng,ở ghép 2 người nam</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>4 triệu/tháng</t>
+          <t>1,75 triệu/tháng</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất cao cấp</t>
         </is>
       </c>
       <c r="F46" t="n">
         <v>0</v>
       </c>
       <c r="G46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H46" t="n">
         <v>0</v>
@@ -2456,34 +2456,34 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/127354068.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129197063.htm</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CHO THUÊ PHÒNG TRỌ – MẶT TIỀN ĐƯỜNG – GẦN NHIỀU TRƯỜNG ĐẠI HỌC</t>
+          <t>Cho Thuê Phòng Thoáng Mát</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2,5 triệu/tháng</t>
+          <t>3,9 triệu/tháng</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>37 m²</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F47" t="n">
@@ -2500,14 +2500,14 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129139688.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129191886.htm</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Cho Thuê Phòng Trọ Cao cấp!</t>
+          <t>Cho thuê phòng trọ</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2517,17 +2517,17 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>18 m²</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F48" t="n">
@@ -2537,41 +2537,41 @@
         <v>0</v>
       </c>
       <c r="H48" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I48" t="n">
         <v>0</v>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128762155.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129166725.htm</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>PHÒNG TRỌ GIÁ RẺ HÒA XUÂN , CẨM LỆ ĐÀ NẴNG</t>
+          <t>💥💥💥💥💥Còn trống 1 phòng ***</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>1,5 triệu/tháng</t>
+          <t>3,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>28 m²</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F49" t="n">
@@ -2584,28 +2584,28 @@
         <v>1</v>
       </c>
       <c r="I49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129151785.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128498042.htm</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Phòng sạch mới ken- wc riêng - tắm riêng</t>
+          <t>CHO THUÊ CĂN HỘ MỚI XÂY 100% - SỐ 17 CỒN DẦU 19 - HÒA XUÂN - CẨM LỆ</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>1,8 triệu/tháng</t>
+          <t>4,8 triệu/tháng</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>21 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2615,11 +2615,11 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G50" t="n">
         <v>0</v>
@@ -2632,38 +2632,38 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129120249.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128248490.htm</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Căn hộ 1 , 2 PN khu vực Mỹ Khê - full nội thất</t>
+          <t>Cho thuê phòng đủ nội thất gần Đại học FPT, giá sinh viên</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>13 triệu/tháng</t>
+          <t>4 triệu/tháng</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>55 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G51" t="n">
         <v>0</v>
@@ -2676,14 +2676,14 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129132617.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/127354068.htm</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Cho thuê trọ gác lửng bạn công</t>
+          <t>CHO THUÊ PHÒNG TRỌ – MẶT TIỀN ĐƯỜNG – GẦN NHIỀU TRƯỜNG ĐẠI HỌC</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2693,12 +2693,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>22 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2716,28 +2716,28 @@
         <v>0</v>
       </c>
       <c r="I52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129123911.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129139688.htm</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CHO THUÊ PHÒNG TRONG NHÀ NGUYÊN CĂN</t>
+          <t>Cho Thuê Phòng Trọ Cao cấp!</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>1,5 triệu/tháng</t>
+          <t>2,2 triệu/tháng</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>10 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2757,41 +2757,41 @@
         <v>0</v>
       </c>
       <c r="H53" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I53" t="n">
         <v>0</v>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129141283.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128762155.htm</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CHO THUÊ PHÒNG TRỌ NGAY PHỐ ĐI BỘ ĐƯỜNG AN THƯỢNG 2</t>
+          <t>PHÒNG TRỌ GIÁ RẺ HÒA XUÂN , CẨM LỆ ĐÀ NẴNG</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2,5 triệu/tháng</t>
+          <t>1,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>16 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F54" t="n">
@@ -2801,26 +2801,26 @@
         <v>0</v>
       </c>
       <c r="H54" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I54" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129137717.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129151785.htm</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Phòng trọ 21m2 đường Bùi Chát- quận Liên Chiểu</t>
+          <t>Phòng sạch mới ken- wc riêng - tắm riêng</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>1,6 triệu/tháng</t>
+          <t>1,8 triệu/tháng</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2830,7 +2830,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2852,68 +2852,68 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129129385.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129120249.htm</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>MỜI THUE TRỌ</t>
+          <t>Căn hộ 1 , 2 PN khu vực Mỹ Khê - full nội thất</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2 triệu/tháng</t>
+          <t>13 triệu/tháng</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>15 m²</t>
+          <t>55 m²</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F56" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G56" t="n">
         <v>0</v>
       </c>
       <c r="H56" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I56" t="n">
         <v>0</v>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129128838.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129132617.htm</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Cho thuê phòng HOTEL gần Crowne, FPT, BV 600 giường,...</t>
+          <t>Cho thuê trọ gác lửng bạn công</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>3,3 triệu/tháng</t>
+          <t>2,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>32 m²</t>
+          <t>22 m²</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2923,7 +2923,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F57" t="n">
@@ -2933,41 +2933,41 @@
         <v>0</v>
       </c>
       <c r="H57" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I57" t="n">
         <v>1</v>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129112267.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129123911.htm</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Cho thuê nhà nguyên căn</t>
+          <t>CHO THUÊ PHÒNG TRONG NHÀ NGUYÊN CĂN</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>1,3 triệu/tháng</t>
+          <t>1,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>13 m²</t>
+          <t>10 m²</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F58" t="n">
@@ -2984,107 +2984,107 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129125566.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129141283.htm</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>[𝗛𝗔̉𝗜 𝗖𝗛𝗔̂𝗨] 𝗣𝗵𝗼̀𝗻𝗴 𝗙𝘂𝗹𝗹 𝗡𝗼̣̂𝗶 𝗧𝗵𝗮̂́𝘁 𝗠𝗼̛́𝗶</t>
+          <t>CHO THUÊ PHÒNG TRỌ NGAY PHỐ ĐI BỘ ĐƯỜNG AN THƯỢNG 2</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>3,4 triệu/tháng</t>
+          <t>2,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>16 m²</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F59" t="n">
         <v>0</v>
       </c>
       <c r="G59" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H59" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I59" t="n">
         <v>1</v>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129122293.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129137717.htm</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>cho thuê nhà mặt tiền trung tâm , ngay nguyễn phước lan</t>
+          <t>Phòng trọ 21m2 đường Bùi Chát- quận Liên Chiểu</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>4 triệu/tháng</t>
+          <t>1,6 triệu/tháng</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>21 m²</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F60" t="n">
         <v>0</v>
       </c>
       <c r="G60" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H60" t="n">
         <v>0</v>
       </c>
       <c r="I60" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129121298.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129129385.htm</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Phòng trọ tiện nghi, trung tâm Ngũ Hành Sơn</t>
+          <t>MỜI THUE TRỌ</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2,5 triệu/tháng</t>
+          <t>2 triệu/tháng</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3094,7 +3094,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -3103,7 +3103,7 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G61" t="n">
         <v>0</v>
@@ -3112,33 +3112,33 @@
         <v>1</v>
       </c>
       <c r="I61" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128189660.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129128838.htm</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Phòng vip cho thuê giá rẻ</t>
+          <t>Cho thuê phòng HOTEL gần Crowne, FPT, BV 600 giường,...</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>3 triệu/tháng</t>
+          <t>3,3 triệu/tháng</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>35 m²</t>
+          <t>32 m²</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -3153,80 +3153,80 @@
         <v>0</v>
       </c>
       <c r="H62" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I62" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129080805.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129112267.htm</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>cho thuê phòng trọ quận thanh khê</t>
+          <t>Cho thuê nhà nguyên căn</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>3 triệu/tháng</t>
+          <t>1,3 triệu/tháng</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>13 m²</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F63" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G63" t="n">
         <v>0</v>
       </c>
       <c r="H63" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I63" t="n">
         <v>0</v>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129096348.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129125566.htm</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ đường Tô Hiến Thành</t>
+          <t>[𝗛𝗔̉𝗜 𝗖𝗛𝗔̂𝗨] 𝗣𝗵𝗼̀𝗻𝗴 𝗙𝘂𝗹𝗹 𝗡𝗼̣̂𝗶 𝗧𝗵𝗮̂́𝘁 𝗠𝗼̛́𝗶</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2,5 triệu/tháng</t>
+          <t>3,4 triệu/tháng</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>19 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -3238,48 +3238,48 @@
         <v>0</v>
       </c>
       <c r="G64" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H64" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I64" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129104381.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129122293.htm</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Cho thuê phòng diện tích 20m2 trên đường Hoàng Đức Lương, An Hải Bắc</t>
+          <t>cho thuê nhà mặt tiền trung tâm , ngay nguyễn phước lan</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>3,3 triệu/tháng</t>
+          <t>4 triệu/tháng</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F65" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G65" t="n">
         <v>1</v>
@@ -3292,24 +3292,24 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/127435716.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129121298.htm</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Cho thuê căn hộ đầy đủ nội thất gần Đh Fpt, Việt Hàn</t>
+          <t>Phòng trọ tiện nghi, trung tâm Ngũ Hành Sơn</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>3 triệu/tháng</t>
+          <t>2,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>15 m²</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -3319,51 +3319,51 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F66" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G66" t="n">
         <v>0</v>
       </c>
       <c r="H66" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I66" t="n">
         <v>1</v>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128764556.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128189660.htm</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>cho thuê phòng trọ, thanh vinh 900k, 109/116/10 phạm như xương 1,200k</t>
+          <t>Phòng vip cho thuê giá rẻ</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>900000 đ/tháng</t>
+          <t>3 triệu/tháng</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>35 m²</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F67" t="n">
@@ -3380,29 +3380,29 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129088217.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129080805.htm</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CHỈ TỪ 1TR850/THÁNG VỚI CHỖ Ở ĐẦY ĐỦ TIỆN NGHI CHO 1 NGƯỜI</t>
+          <t>cho thuê phòng trọ quận thanh khê</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>1,85 triệu/tháng</t>
+          <t>3 triệu/tháng</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>10 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -3411,7 +3411,7 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G68" t="n">
         <v>0</v>
@@ -3420,38 +3420,38 @@
         <v>1</v>
       </c>
       <c r="I68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129071161.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129096348.htm</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Phòng đầy đủ tiện nghi chỉ vào ở</t>
+          <t>Cho thuê phòng trọ đường Tô Hiến Thành</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>3 triệu/tháng</t>
+          <t>2,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>19 m²</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Nội thất cao cấp</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F69" t="n">
@@ -3468,29 +3468,29 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128711543.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129104381.htm</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Cho thuê 3 phòng trọ Kiệt Nguyễn Xuân Hữu</t>
+          <t>Cho thuê phòng diện tích 20m2 trên đường Hoàng Đức Lương, An Hải Bắc</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2,2 triệu/tháng</t>
+          <t>3,3 triệu/tháng</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>100 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -3499,47 +3499,47 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G70" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H70" t="n">
         <v>0</v>
       </c>
       <c r="I70" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129082151.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/127435716.htm</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Phòng Trọ Cho Thuê Rộng</t>
+          <t>Cho thuê căn hộ đầy đủ nội thất gần Đh Fpt, Việt Hàn</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2,5 triệu/tháng</t>
+          <t>3 triệu/tháng</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>35 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F71" t="n">
@@ -3556,34 +3556,34 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129081900.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128764556.htm</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>🔥Hot! Phòng VIP đối diện bãi biển Nguyễn Tất Thành</t>
+          <t>cho thuê phòng trọ, thanh vinh 900k, 109/116/10 phạm như xương 1,200k</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>7 triệu/tháng</t>
+          <t>900000 đ/tháng</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Nội thất cao cấp</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F72" t="n">
@@ -3600,34 +3600,34 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129077873.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129088217.htm</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>🔥Phòng VIP full nội thất view balcon gần bãi biển Mỹ Khuê</t>
+          <t>CHỈ TỪ 1TR850/THÁNG VỚI CHỖ Ở ĐẦY ĐỦ TIỆN NGHI CHO 1 NGƯỜI</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>5,5 triệu/tháng</t>
+          <t>1,85 triệu/tháng</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>10 m²</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Nội thất cao cấp</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F73" t="n">
@@ -3637,36 +3637,36 @@
         <v>0</v>
       </c>
       <c r="H73" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I73" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129077553.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129071161.htm</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Căn hộ full nội thất Hòa Cường Bắc</t>
+          <t>Phòng đầy đủ tiện nghi chỉ vào ở</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>5,5 triệu/tháng</t>
+          <t>3 triệu/tháng</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3675,7 +3675,7 @@
         </is>
       </c>
       <c r="F74" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G74" t="n">
         <v>0</v>
@@ -3688,29 +3688,29 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128138926.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128711543.htm</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ truyền thống tại 06 Nguyễn Khắc Nhu Hoà Minh</t>
+          <t>Cho thuê 3 phòng trọ Kiệt Nguyễn Xuân Hữu</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>1,8 triệu/tháng</t>
+          <t>2,2 triệu/tháng</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>100 m²</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3732,34 +3732,34 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129042993.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129082151.htm</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ</t>
+          <t>Phòng Trọ Cho Thuê Rộng</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>3 triệu/tháng</t>
+          <t>2,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>35 m²</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Nội thất cao cấp</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F76" t="n">
@@ -3772,38 +3772,38 @@
         <v>0</v>
       </c>
       <c r="I76" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129038584.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129081900.htm</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>phòng trọ 43m2,1 tủ có thể kê thêm tiện ích nếu cần</t>
+          <t>🔥Hot! Phòng VIP đối diện bãi biển Nguyễn Tất Thành</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>3,5 triệu/tháng</t>
+          <t>7 triệu/tháng</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>43 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất cao cấp</t>
         </is>
       </c>
       <c r="F77" t="n">
@@ -3820,34 +3820,34 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129034786.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129077873.htm</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Phòng đầy đủ nội thất thoáng mát CMT8 gần UBND Cẩm Lệ</t>
+          <t>🔥Phòng VIP full nội thất view balcon gần bãi biển Mỹ Khuê</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>3 triệu/tháng</t>
+          <t>5,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>22 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nội thất cao cấp</t>
         </is>
       </c>
       <c r="F78" t="n">
@@ -3860,23 +3860,23 @@
         <v>0</v>
       </c>
       <c r="I78" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129057766.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129077553.htm</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Chính chủ cho thuê phòng 1.7tr/ tháng đã bao điện nước tại Cầu Rồng</t>
+          <t>Căn hộ full nội thất Hòa Cường Bắc</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>1,7 triệu/tháng</t>
+          <t>5,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -3886,56 +3886,56 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nội thất cao cấp</t>
         </is>
       </c>
       <c r="F79" t="n">
         <v>1</v>
       </c>
       <c r="G79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H79" t="n">
         <v>0</v>
       </c>
       <c r="I79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129043372.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128138926.htm</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Cho Thuê phòng trọ gần Trung tâm Liên Chiểu</t>
+          <t>Cho thuê phòng trọ</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2 triệu/tháng</t>
+          <t>3 triệu/tháng</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất cao cấp</t>
         </is>
       </c>
       <c r="F80" t="n">
@@ -3952,24 +3952,24 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128960732.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129038584.htm</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Căn hộ 1 phòng ngủ 50m2 - Hải Châu Đà Nẵng</t>
+          <t>phòng trọ 43m2,1 tủ có thể kê thêm tiện ích nếu cần</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>6,5 triệu/tháng</t>
+          <t>3,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>50 m²</t>
+          <t>43 m²</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -3979,14 +3979,14 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Nội thất cao cấp</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F81" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G81" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H81" t="n">
         <v>0</v>
@@ -3996,34 +3996,34 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128988916.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129034786.htm</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CHO THUÊ CĂN HỘ MỚI GẦN BÃI BIỂN MỸ AN - KHÔNG GIAN YÊN TĨNH</t>
+          <t>Phòng đầy đủ nội thất thoáng mát CMT8 gần UBND Cẩm Lệ</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>6,3 triệu/tháng</t>
+          <t>3 triệu/tháng</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>22 m²</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Nội thất cao cấp</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F82" t="n">
@@ -4036,133 +4036,133 @@
         <v>0</v>
       </c>
       <c r="I82" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128991832.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129057766.htm</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Cần nam ở ghép nhà rộng rãi tại đầu đường Tôn Đản, có đầy đủ tiện nghi</t>
+          <t>Chính chủ cho thuê phòng 1.7tr/ tháng đã bao điện nước tại Cầu Rồng</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>1 triệu/tháng</t>
+          <t>1,7 triệu/tháng</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>79 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F83" t="n">
         <v>1</v>
       </c>
       <c r="G83" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H83" t="n">
         <v>0</v>
       </c>
       <c r="I83" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128099349.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129043372.htm</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Phòng trọ mới , đường rộng ngây cầu nguyễn tri phương</t>
+          <t>Căn hộ 1 phòng ngủ 50m2 - Hải Châu Đà Nẵng</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>3,6 triệu/tháng</t>
+          <t>6,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>50 m²</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nội thất cao cấp</t>
         </is>
       </c>
       <c r="F84" t="n">
         <v>1</v>
       </c>
       <c r="G84" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H84" t="n">
         <v>0</v>
       </c>
       <c r="I84" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129001680.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128988916.htm</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>MỜI BẠN VỀ NHÀ</t>
+          <t>CHO THUÊ CĂN HỘ MỚI GẦN BÃI BIỂN MỸ AN - KHÔNG GIAN YÊN TĨNH</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>7 triệu/tháng</t>
+          <t>6,3 triệu/tháng</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>68.8 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nội thất cao cấp</t>
         </is>
       </c>
       <c r="F85" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G85" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H85" t="n">
         <v>0</v>
@@ -4172,29 +4172,29 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128979633.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128991832.htm</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ gần trường Đại học FPT, Việt Hàn...</t>
+          <t>Cần nam ở ghép nhà rộng rãi tại đầu đường Tôn Đản, có đầy đủ tiện nghi</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>1,5 triệu/tháng</t>
+          <t>1 triệu/tháng</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>79 m²</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -4203,7 +4203,7 @@
         </is>
       </c>
       <c r="F86" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G86" t="n">
         <v>0</v>
@@ -4216,29 +4216,29 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128980753.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128099349.htm</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>cho thuê giường dorm</t>
+          <t>Phòng trọ mới , đường rộng ngây cầu nguyễn tri phương</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>1,4 triệu/tháng</t>
+          <t>3,6 triệu/tháng</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>38 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -4250,29 +4250,29 @@
         <v>1</v>
       </c>
       <c r="G87" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H87" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I87" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/126893939.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129001680.htm</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>GÁC LỬNG CHO THUÊ GẦN CẦU HÒA XUÂN</t>
+          <t>Cho thuê phòng trọ gần trường Đại học FPT, Việt Hàn...</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>4,3 triệu/tháng</t>
+          <t>1,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -4282,7 +4282,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -4304,29 +4304,29 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128974469.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128980753.htm</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ kiệt Hà Huy Tập - Đà Nẵng</t>
+          <t>GÁC LỬNG CHO THUÊ GẦN CẦU HÒA XUÂN</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2,4 triệu/tháng</t>
+          <t>4,3 triệu/tháng</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>15 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -4335,7 +4335,7 @@
         </is>
       </c>
       <c r="F89" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G89" t="n">
         <v>0</v>
@@ -4344,33 +4344,33 @@
         <v>0</v>
       </c>
       <c r="I89" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128972748.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128974469.htm</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Cho thuê Căn Hộ 50m2 1 phòng ngủ đủ nội thất đườg Lê Thanh Nghị</t>
+          <t>Cho thuê phòng trọ kiệt Hà Huy Tập - Đà Nẵng</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>5,9 triệu/tháng</t>
+          <t>2,4 triệu/tháng</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>50 m²</t>
+          <t>15 m²</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -4382,7 +4382,7 @@
         <v>1</v>
       </c>
       <c r="G90" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H90" t="n">
         <v>0</v>
@@ -4392,29 +4392,29 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128960894.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128972748.htm</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ giá rẻ 41 Nguyễn Xuân Hữu, gần Ông Ích Đường, CMT8</t>
+          <t>Cho thuê Căn Hộ 50m2 1 phòng ngủ đủ nội thất đườg Lê Thanh Nghị</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>1,7 triệu/tháng</t>
+          <t>5,9 triệu/tháng</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>50 m²</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -4423,20 +4423,20 @@
         </is>
       </c>
       <c r="F91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H91" t="n">
         <v>0</v>
       </c>
       <c r="I91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/126547864.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128960894.htm</t>
         </is>
       </c>
     </row>
@@ -7121,50 +7121,6 @@
       <c r="J152" t="inlineStr">
         <is>
           <t>https://www.nhatot.com/cho-thue-phong-tro/127976873.htm</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t>cần thuê nhà</t>
-        </is>
-      </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>2 triệu/tháng</t>
-        </is>
-      </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>30 m²</t>
-        </is>
-      </c>
-      <c r="D153" t="inlineStr">
-        <is>
-          <t>Huyện Hòa Vang, Đà Nẵng</t>
-        </is>
-      </c>
-      <c r="E153" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F153" t="n">
-        <v>0</v>
-      </c>
-      <c r="G153" t="n">
-        <v>0</v>
-      </c>
-      <c r="H153" t="n">
-        <v>0</v>
-      </c>
-      <c r="I153" t="n">
-        <v>0</v>
-      </c>
-      <c r="J153" t="inlineStr">
-        <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/127973425.htm</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto scrape + SQL (from Excel) 2025-11-26 17:16:26
</commit_message>
<xml_diff>
--- a/nhatot_phongtro_danang_all.xlsx
+++ b/nhatot_phongtro_danang_all.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J151"/>
+  <dimension ref="A1:J149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -483,12 +483,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>phòng Cho Thuê  tầng  2 - cửa sổ ban công thoáng mát</t>
+          <t>PHÒNG CHO THUÊ CAO CẤP - TRUNG TÂM TP</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2,8 triệu/tháng</t>
+          <t>2,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -498,12 +498,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -513,41 +513,41 @@
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/127699774.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129322964.htm</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ (FPT, VKU, Làng Đại học)</t>
+          <t>Cho thuê phòng trọ.cho nữ thuê.phòng mới.gác lửng.đ/c 11 lê sao</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>950000 đ/tháng</t>
+          <t>1,9 triệu/tháng</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>16 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -557,80 +557,80 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129300791.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129320030.htm</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ.cho nữ thuê.đ.c 11 lê sao.phòng giữa</t>
+          <t>phòng trong nhà mặt tiền hoàng diệu</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1,9 triệu/tháng</t>
+          <t>3,3 triệu/tháng</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129298631.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128458947.htm</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MỜI BẠN VỀ NHÀ</t>
+          <t>phòng Cho Thuê  tầng  2 - cửa sổ ban công thoáng mát</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>7 triệu/tháng</t>
+          <t>2,8 triệu/tháng</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>68.8 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -639,37 +639,37 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128979633.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/127699774.htm</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PHÒNG ĐẦY ĐỦ TIỆN NGHI NGŨ HÀNH SƠN ĐÀ NẴNG</t>
+          <t>phòng trọ Ngũ Hành Sơn đối diện chợ Bắc Mỹ An, gần Đại học Kinh tế</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2,99 triệu/tháng</t>
+          <t>3,2 triệu/tháng</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>18 m²</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -679,183 +679,183 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F6" t="n">
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H6" t="n">
         <v>1</v>
       </c>
       <c r="I6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128928025.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129280652.htm</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Căn hộ mini full nội thất Sơn Trà</t>
+          <t>🏡 BÁN DÃY TRỌ 5 PHÒNG KIỆT ÔTÔ 151 ÂU CƠ - TRUNG TÂM HÒA KHÁNH</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>3,8 triệu/tháng</t>
+          <t>3,5 tỷ/tháng</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>120 m²</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128837798.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129287916.htm</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>cho thuê giường dorm</t>
+          <t>Sau lưng sân bóng Ông Bầu, gần ngã tư 29/3 &amp; Võ Chí Công – Hoà Xuân</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1,4 triệu/tháng</t>
+          <t>3,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>38 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G8" t="n">
         <v>1</v>
       </c>
       <c r="H8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/126893939.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129288253.htm</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>cho thuê dorm - sleep box</t>
+          <t>Phòng ngoài cùng có cửa sổ 12m2 An Hải Bắc, Sơn Trà Đà Nẵng</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>1,8 triệu/tháng</t>
+          <t>1,6 triệu/tháng</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10 m²</t>
+          <t>12 m²</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Nội thất cao cấp</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129289834.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129284531.htm</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>139 ngô quyền CHO THUÊ PHÒNG TRỌ</t>
+          <t>Phòng trọ đường ôto không ngập</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>1,7 triệu/tháng</t>
+          <t>2,2 triệu/tháng</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất cao cấp</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -865,36 +865,36 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129289097.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129306812.htm</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Sau lưng sân bóng Ông Bầu, gần ngã tư 29/3 &amp; Võ Chí Công – Hoà Xuân</t>
+          <t>Cho thuê phòng gần bến xe , FPT, sư phạm , duy tân , bách khoa</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>3,5 triệu/tháng</t>
+          <t>1,4 triệu/tháng</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -906,44 +906,44 @@
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129288253.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128382768.htm</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>🏡 BÁN DÃY TRỌ 5 PHÒNG KIỆT ÔTÔ 151 ÂU CƠ - TRUNG TÂM HÒA KHÁNH</t>
+          <t>Cho thuê phòng Xịn giá rẻ ở Cẩm Lệ</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>3,5 tỷ/tháng</t>
+          <t>3 triệu/tháng</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>120 m²</t>
+          <t>40 m²</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -960,24 +960,24 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129287916.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128635113.htm</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Phòng trọ full nội thất 25m2, 55 Thủy Sơn 5 - Hòa Hải - Ngủ Hành Sơn</t>
+          <t>Cho thuê phòng trọ (FPT, VKU, Làng Đại học)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2,4 triệu/tháng</t>
+          <t>950000 đ/tháng</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>16 m²</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -987,58 +987,58 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129285329.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129300791.htm</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Phòng ngoài cùng có cửa sổ 12m2 An Hải Bắc, Sơn Trà Đà Nẵng</t>
+          <t>MỜI BẠN VỀ NHÀ</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1,6 triệu/tháng</t>
+          <t>7 triệu/tháng</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>12 m²</t>
+          <t>68.8 m²</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -1048,38 +1048,38 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129284531.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128979633.htm</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>phòng trọ cao cấp</t>
+          <t>Căn hộ mini full nội thất Sơn Trà</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>3 triệu/tháng</t>
+          <t>3,8 triệu/tháng</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>27 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G15" t="n">
         <v>1</v>
@@ -1088,45 +1088,45 @@
         <v>1</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/127030626.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128837798.htm</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>phòng trọ Ngũ Hành Sơn đối diện chợ Bắc Mỹ An, gần Đại học Kinh tế</t>
+          <t>cho thuê giường dorm</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>3,2 triệu/tháng</t>
+          <t>1,4 triệu/tháng</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>18 m²</t>
+          <t>38 m²</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H16" t="n">
         <v>1</v>
@@ -1136,63 +1136,63 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129280652.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/126893939.htm</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Phòng trọ ngay cầu rồng hướng ra biển, giá 2,9tr</t>
+          <t>cho thuê dorm - sleep box</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2,9 triệu/tháng</t>
+          <t>1,8 triệu/tháng</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>15 m²</t>
+          <t>10 m²</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất cao cấp</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129279640.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129289834.htm</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ</t>
+          <t>139 ngô quyền CHO THUÊ PHÒNG TRỌ</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2 triệu/tháng</t>
+          <t>1,7 triệu/tháng</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1202,12 +1202,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F18" t="n">
@@ -1217,85 +1217,85 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I18" t="n">
         <v>0</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129278299.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129289097.htm</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Phòng trọ nhỏ giá cả hợp lí đường Nguyễn Công Trứ gần cầu Rồng</t>
+          <t>phòng trọ cao cấp</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2,9 triệu/tháng</t>
+          <t>3 triệu/tháng</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>15 m²</t>
+          <t>27 m²</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/127178277.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/127030626.htm</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CHO THUÊ PHÒNG TRỌ SẠCH SẼ MÁT MẺ TRONG NHÀ 4 TẦNG KHU VỰC THANH KHÊ</t>
+          <t>Phòng trọ ngay cầu rồng hướng ra biển, giá 2,9tr</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>1,8 triệu/tháng</t>
+          <t>2,9 triệu/tháng</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>15 m²</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F20" t="n">
@@ -1305,36 +1305,36 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I20" t="n">
         <v>0</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129251296.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129279640.htm</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Cho thuê phòng đầy đủ tiện nghi,khu ngã ba huế,bến xe</t>
+          <t>Cho thuê phòng trọ</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>1,8 triệu/tháng</t>
+          <t>2 triệu/tháng</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>15 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1343,10 +1343,10 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H21" t="n">
         <v>0</v>
@@ -1356,38 +1356,38 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128606799.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129278299.htm</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>TRỌ GÁC LỬNG 25M2 CHỈ 1.8TR TRONG MẶT TIỀN KIỀU PHỤNG RIÊNG CHỦ</t>
+          <t>Phòng trọ nhỏ giá cả hợp lí đường Nguyễn Công Trứ gần cầu Rồng</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>5 triệu/tháng</t>
+          <t>2,9 triệu/tháng</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>15 m²</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
@@ -1396,42 +1396,42 @@
         <v>0</v>
       </c>
       <c r="I22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129266347.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/127178277.htm</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>phòng trong nhà mặt tiền hoàng diệu</t>
+          <t>CHO THUÊ PHÒNG TRỌ SẠCH SẼ MÁT MẺ TRONG NHÀ 4 TẦNG KHU VỰC THANH KHÊ</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>3,3 triệu/tháng</t>
+          <t>1,8 triệu/tháng</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G23" t="n">
         <v>0</v>
@@ -1444,41 +1444,41 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128458947.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129251296.htm</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Nhà nguyên căn, dt 100m2, 234/10 Đỗ Bá</t>
+          <t>Cho thuê phòng đầy đủ tiện nghi,khu ngã ba huế,bến xe</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>7 triệu/tháng</t>
+          <t>1,8 triệu/tháng</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>100 m²</t>
+          <t>15 m²</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H24" t="n">
         <v>0</v>
@@ -1488,14 +1488,14 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129258007.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128606799.htm</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Cho thuê nguyên tầng 3, diện tích 100m2</t>
+          <t>TRỌ GÁC LỬNG 25M2 CHỈ 1.8TR TRONG MẶT TIỀN KIỀU PHỤNG RIÊNG CHỦ</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1505,21 +1505,21 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>100 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G25" t="n">
         <v>0</v>
@@ -1528,33 +1528,33 @@
         <v>0</v>
       </c>
       <c r="I25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129257747.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129266347.htm</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Phòng trọ nội thất cơ bản</t>
+          <t>Nhà nguyên căn, dt 100m2, 234/10 Đỗ Bá</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2,5 triệu/tháng</t>
+          <t>7 triệu/tháng</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>18 m²</t>
+          <t>100 m²</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1563,47 +1563,47 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G26" t="n">
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129239038.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129258007.htm</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Nhà trọ sang chảnh</t>
+          <t>Cho thuê nguyên tầng 3, diện tích 100m2</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2,7 triệu/tháng</t>
+          <t>5 triệu/tháng</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>17 m²</t>
+          <t>100 m²</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F27" t="n">
@@ -1616,116 +1616,116 @@
         <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/127668535.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129257747.htm</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Nhà trọ Văn Minh có 1 phòng trống</t>
+          <t>Phòng trọ nội thất cơ bản</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2,2 triệu/tháng</t>
+          <t>2,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>18 m²</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G28" t="n">
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129229044.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129239038.htm</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>cho thuê phòng trọ phường Hải Châu</t>
+          <t>Nhà trọ sang chảnh</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>3,5 triệu/tháng</t>
+          <t>2,7 triệu/tháng</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>32 m²</t>
+          <t>17 m²</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F29" t="n">
         <v>1</v>
       </c>
       <c r="G29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129246849.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/127668535.htm</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ (Chung chủ)</t>
+          <t>Nhà trọ Văn Minh có 1 phòng trống</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>3 triệu/tháng</t>
+          <t>2,2 triệu/tháng</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F30" t="n">
@@ -1752,78 +1752,78 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129246276.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129229044.htm</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ tại 508 Lê Văn Hiến, Ngũ Hành Sơn, TP. Đà Nẵng</t>
+          <t>cho thuê phòng trọ phường Hải Châu</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>1,5 triệu/tháng</t>
+          <t>3,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>32 m²</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129243560.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129246849.htm</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ rộng rãi, an ninh, gần các trường học</t>
+          <t>Cho thuê phòng trọ (Chung chủ)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2,4 triệu/tháng</t>
+          <t>3 triệu/tháng</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F32" t="n">
@@ -1836,28 +1836,28 @@
         <v>0</v>
       </c>
       <c r="I32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129237617.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129246276.htm</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Phòng ban công full nội thất new 100% khu FPT - Ngũ Hành Sơn</t>
+          <t>Cho thuê phòng trọ tại 508 Lê Văn Hiến, Ngũ Hành Sơn, TP. Đà Nẵng</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>4 triệu/tháng</t>
+          <t>1,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>40 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1867,55 +1867,55 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G33" t="n">
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128629777.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129243560.htm</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Phòng Full Nội Thất Khu FPT - Ngũ Hành Sơn</t>
+          <t>Cho thuê phòng trọ rộng rãi, an ninh, gần các trường học</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>3,9 triệu/tháng</t>
+          <t>2,2 triệu/tháng</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>40 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G34" t="n">
         <v>0</v>
@@ -1924,33 +1924,33 @@
         <v>0</v>
       </c>
       <c r="I34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128025078.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129237617.htm</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>phòng cho thuê trọ</t>
+          <t>Phòng ban công full nội thất new 100% khu FPT - Ngũ Hành Sơn</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>3,6 triệu/tháng</t>
+          <t>4 triệu/tháng</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>28 m²</t>
+          <t>40 m²</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1962,39 +1962,39 @@
         <v>1</v>
       </c>
       <c r="G35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H35" t="n">
         <v>1</v>
       </c>
       <c r="I35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129192954.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128629777.htm</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Cho thuê phòng full option. 129  Nguyễn Khánh Toàn Trung Tâm Đà Nẵng</t>
+          <t>Phòng Full Nội Thất Khu FPT - Ngũ Hành Sơn</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>4,3 triệu/tháng</t>
+          <t>3,9 triệu/tháng</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>40 m²</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2006,34 +2006,34 @@
         <v>1</v>
       </c>
       <c r="G36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I36" t="n">
         <v>0</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128845940.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128025078.htm</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Cho Thuê trọ phòng khách sạn</t>
+          <t>phòng cho thuê trọ</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>3,5 triệu/tháng</t>
+          <t>3,6 triệu/tháng</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>28 m²</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2050,83 +2050,83 @@
         <v>1</v>
       </c>
       <c r="G37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I37" t="n">
         <v>0</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/127808442.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129192954.htm</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Phòng trọ 17m2 Đường Lương Thế Vinh Quận Sơn Trà</t>
+          <t>Cho thuê phòng full option. 129  Nguyễn Khánh Toàn Trung Tâm Đà Nẵng</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>3 triệu/tháng</t>
+          <t>4,3 triệu/tháng</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>17 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I38" t="n">
         <v>0</v>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129201071.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128845940.htm</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>căn hộ tại 240/6 lê duẩn</t>
+          <t>Cho Thuê trọ phòng khách sạn</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>3 triệu/tháng</t>
+          <t>3,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>18 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2135,7 +2135,7 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G39" t="n">
         <v>0</v>
@@ -2148,24 +2148,24 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129220491.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/127808442.htm</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Phòng trọ 35mv đg Ng Trung Trực - cách Sông Hàn 1km- gần tr Greenwich</t>
+          <t>Phòng trọ 17m2 Đường Lương Thế Vinh Quận Sơn Trà</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>3,5 triệu/tháng</t>
+          <t>3 triệu/tháng</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>35 m²</t>
+          <t>17 m²</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F40" t="n">
@@ -2192,34 +2192,34 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129229623.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129201071.htm</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ 1tr5</t>
+          <t>căn hộ tại 240/6 lê duẩn</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>1,5 triệu/tháng</t>
+          <t>3 triệu/tháng</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>18 m²</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F41" t="n">
@@ -2232,82 +2232,82 @@
         <v>0</v>
       </c>
       <c r="I41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129225686.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129220491.htm</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ đường Châu Văn Liêm, gần Vũ Trường Phương Đông</t>
+          <t>Phòng trọ 35mv đg Ng Trung Trực - cách Sông Hàn 1km- gần tr Greenwich</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>3,7 triệu/tháng</t>
+          <t>3,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>32 m²</t>
+          <t>35 m²</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Nội thất cao cấp</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G42" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H42" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I42" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128605782.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129229623.htm</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Trống 1 căn , full nội thất , phòng ngủ tách biệt</t>
+          <t>Cho thuê phòng trọ 1tr5</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>4,1 triệu/tháng</t>
+          <t>1,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>40 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F43" t="n">
@@ -2320,77 +2320,77 @@
         <v>0</v>
       </c>
       <c r="I43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129218959.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129225686.htm</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Cho thuê phòng mặt tiền 68/20 Nguyễn mộng tuân ngay bến xe</t>
+          <t>Cho thuê phòng trọ đường Châu Văn Liêm, gần Vũ Trường Phương Đông</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>4 triệu/tháng</t>
+          <t>3,7 triệu/tháng</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>32 m²</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất cao cấp</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129217669.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128605782.htm</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Phòng trọ cho người độc thân tại sơn trà</t>
+          <t>Trống 1 căn , full nội thất , phòng ngủ tách biệt</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>1,7 triệu/tháng</t>
+          <t>4,1 triệu/tháng</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>400 m²</t>
+          <t>40 m²</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2412,38 +2412,38 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/125998127.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129218959.htm</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>phòng trọ gần cầu hoà xuân</t>
+          <t>Cho thuê phòng mặt tiền 68/20 Nguyễn mộng tuân ngay bến xe</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>6 triệu/tháng</t>
+          <t>4 triệu/tháng</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>40 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G46" t="n">
         <v>0</v>
@@ -2456,34 +2456,34 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129199929.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129217669.htm</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Phòng mới rộng đẹp Hoà Phú 27 Hoà Minh Liên Chiểu.</t>
+          <t>Phòng trọ cho người độc thân tại sơn trà</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>4,5 triệu/tháng</t>
+          <t>1,7 triệu/tháng</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>40 m²</t>
+          <t>400 m²</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F47" t="n">
@@ -2500,38 +2500,38 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129183180.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/125998127.htm</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ riêng 68/20 Nguyễn mộng tuân</t>
+          <t>phòng trọ gần cầu hoà xuân</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>4 triệu/tháng</t>
+          <t>6 triệu/tháng</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>40 m²</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G48" t="n">
         <v>0</v>
@@ -2544,38 +2544,38 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128830619.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129199929.htm</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Phòng trọ 30m2 Hoà Xuân, an ninh, không chung chủ</t>
+          <t>Phòng mới rộng đẹp Hoà Phú 27 Hoà Minh Liên Chiểu.</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2,5 triệu/tháng</t>
+          <t>4,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>28 m²</t>
+          <t>40 m²</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F49" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G49" t="n">
         <v>0</v>
@@ -2588,14 +2588,14 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129184894.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129183180.htm</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>✨ Căn hộ mới 100% đi vào hoạt động</t>
+          <t>Cho thuê phòng trọ riêng 68/20 Nguyễn mộng tuân</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2605,65 +2605,65 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F50" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G50" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H50" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I50" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129198937.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128830619.htm</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ full nội thất</t>
+          <t>Phòng trọ 30m2 Hoà Xuân, an ninh, không chung chủ</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>4,5 triệu/tháng</t>
+          <t>2,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>35 m²</t>
+          <t>28 m²</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G51" t="n">
         <v>0</v>
@@ -2676,58 +2676,58 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128820066.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129184894.htm</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CHO THUE PHONG TRO KCN HOA CAM CAM LE DA NANG</t>
+          <t>✨ Căn hộ mới 100% đi vào hoạt động</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>700000 đ/tháng</t>
+          <t>3,8 triệu/tháng</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>14 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129009631.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129198937.htm</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ gia đình</t>
+          <t>Cho thuê phòng trọ full nội thất</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2737,61 +2737,61 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>60 m²</t>
+          <t>35 m²</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F53" t="n">
         <v>0</v>
       </c>
       <c r="G53" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H53" t="n">
         <v>0</v>
       </c>
       <c r="I53" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128786730.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128820066.htm</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>phòng 2 giường riêng .khách sạn sang trọng,ở ghép 2 người nam</t>
+          <t>Cho thuê phòng trọ gia đình</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>1,75 triệu/tháng</t>
+          <t>4,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>60 m²</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Nội thất cao cấp</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F54" t="n">
@@ -2804,45 +2804,45 @@
         <v>0</v>
       </c>
       <c r="I54" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129197063.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128786730.htm</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Cho Thuê Phòng Thoáng Mát</t>
+          <t>phòng 2 giường riêng .khách sạn sang trọng,ở ghép 2 người nam</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>3,9 triệu/tháng</t>
+          <t>1,75 triệu/tháng</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>37 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nội thất cao cấp</t>
         </is>
       </c>
       <c r="F55" t="n">
         <v>0</v>
       </c>
       <c r="G55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H55" t="n">
         <v>0</v>
@@ -2852,34 +2852,34 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129191886.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129197063.htm</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ</t>
+          <t>Cho Thuê Phòng Thoáng Mát</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2,2 triệu/tháng</t>
+          <t>3,9 triệu/tháng</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>18 m²</t>
+          <t>37 m²</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F56" t="n">
@@ -2896,34 +2896,34 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129166725.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129191886.htm</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>💥💥💥💥💥Còn trống 1 phòng ***</t>
+          <t>Cho thuê phòng trọ</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>3,5 triệu/tháng</t>
+          <t>2,2 triệu/tháng</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>28 m²</t>
+          <t>18 m²</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F57" t="n">
@@ -2933,36 +2933,36 @@
         <v>0</v>
       </c>
       <c r="H57" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I57" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128498042.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129166725.htm</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CHO THUÊ CĂN HỘ MỚI XÂY 100% - SỐ 17 CỒN DẦU 19 - HÒA XUÂN - CẨM LỆ</t>
+          <t>💥💥💥💥💥Còn trống 1 phòng ***</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>4,8 triệu/tháng</t>
+          <t>3,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>28 m²</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2971,32 +2971,32 @@
         </is>
       </c>
       <c r="F58" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G58" t="n">
         <v>0</v>
       </c>
       <c r="H58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128248490.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128498042.htm</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Cho thuê phòng đủ nội thất gần Đại học FPT, giá sinh viên</t>
+          <t>CHO THUÊ CĂN HỘ MỚI XÂY 100% - SỐ 17 CỒN DẦU 19 - HÒA XUÂN - CẨM LỆ</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>4 triệu/tháng</t>
+          <t>4,8 triệu/tháng</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -3006,16 +3006,16 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F59" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G59" t="n">
         <v>0</v>
@@ -3028,29 +3028,29 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/127354068.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128248490.htm</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CHO THUÊ PHÒNG TRỌ – MẶT TIỀN ĐƯỜNG – GẦN NHIỀU TRƯỜNG ĐẠI HỌC</t>
+          <t>Cho thuê phòng đủ nội thất gần Đại học FPT, giá sinh viên</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2,5 triệu/tháng</t>
+          <t>4 triệu/tháng</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -3072,19 +3072,19 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129139688.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/127354068.htm</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Cho Thuê Phòng Trọ Cao cấp!</t>
+          <t>CHO THUÊ PHÒNG TRỌ – MẶT TIỀN ĐƯỜNG – GẦN NHIỀU TRƯỜNG ĐẠI HỌC</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2,2 triệu/tháng</t>
+          <t>2,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3094,7 +3094,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -3109,26 +3109,26 @@
         <v>0</v>
       </c>
       <c r="H61" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I61" t="n">
         <v>0</v>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128762155.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129139688.htm</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>PHÒNG TRỌ GIÁ RẺ HÒA XUÂN , CẨM LỆ ĐÀ NẴNG</t>
+          <t>Cho Thuê Phòng Trọ Cao cấp!</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>1,5 triệu/tháng</t>
+          <t>2,2 triệu/tháng</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -3160,24 +3160,24 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129151785.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128762155.htm</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Phòng sạch mới ken- wc riêng - tắm riêng</t>
+          <t>PHÒNG TRỌ GIÁ RẺ HÒA XUÂN , CẨM LỆ ĐÀ NẴNG</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>1,8 triệu/tháng</t>
+          <t>1,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>21 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F63" t="n">
@@ -3197,45 +3197,45 @@
         <v>0</v>
       </c>
       <c r="H63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I63" t="n">
         <v>0</v>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129120249.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129151785.htm</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Căn hộ 1 , 2 PN khu vực Mỹ Khê - full nội thất</t>
+          <t>Phòng sạch mới ken- wc riêng - tắm riêng</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>13 triệu/tháng</t>
+          <t>1,8 triệu/tháng</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>55 m²</t>
+          <t>21 m²</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F64" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G64" t="n">
         <v>0</v>
@@ -3248,38 +3248,38 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129132617.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129120249.htm</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Cho thuê trọ gác lửng bạn công</t>
+          <t>Căn hộ 1 , 2 PN khu vực Mỹ Khê - full nội thất</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2,5 triệu/tháng</t>
+          <t>13 triệu/tháng</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>22 m²</t>
+          <t>55 m²</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G65" t="n">
         <v>0</v>
@@ -3288,33 +3288,33 @@
         <v>0</v>
       </c>
       <c r="I65" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129123911.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129132617.htm</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CHO THUÊ PHÒNG TRONG NHÀ NGUYÊN CĂN</t>
+          <t>Cho thuê trọ gác lửng bạn công</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>1,5 triệu/tháng</t>
+          <t>2,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>10 m²</t>
+          <t>22 m²</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -3332,38 +3332,38 @@
         <v>0</v>
       </c>
       <c r="I66" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129141283.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129123911.htm</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CHO THUÊ PHÒNG TRỌ NGAY PHỐ ĐI BỘ ĐƯỜNG AN THƯỢNG 2</t>
+          <t>CHO THUÊ PHÒNG TRONG NHÀ NGUYÊN CĂN</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2,5 triệu/tháng</t>
+          <t>1,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>16 m²</t>
+          <t>10 m²</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F67" t="n">
@@ -3376,38 +3376,38 @@
         <v>0</v>
       </c>
       <c r="I67" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129137717.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129141283.htm</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Phòng trọ 21m2 đường Bùi Chát- quận Liên Chiểu</t>
+          <t>CHO THUÊ PHÒNG TRỌ NGAY PHỐ ĐI BỘ ĐƯỜNG AN THƯỢNG 2</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>1,6 triệu/tháng</t>
+          <t>2,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>21 m²</t>
+          <t>16 m²</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F68" t="n">
@@ -3420,38 +3420,38 @@
         <v>0</v>
       </c>
       <c r="I68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129129385.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129137717.htm</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>MỜI THUE TRỌ</t>
+          <t>Phòng trọ 21m2 đường Bùi Chát- quận Liên Chiểu</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2 triệu/tháng</t>
+          <t>1,6 triệu/tháng</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>15 m²</t>
+          <t>21 m²</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F69" t="n">
@@ -3461,41 +3461,41 @@
         <v>0</v>
       </c>
       <c r="H69" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I69" t="n">
         <v>0</v>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129128838.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129129385.htm</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Cho thuê phòng HOTEL gần Crowne, FPT, BV 600 giường,...</t>
+          <t>MỜI THUE TRỌ</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>3,3 triệu/tháng</t>
+          <t>2 triệu/tháng</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>32 m²</t>
+          <t>15 m²</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F70" t="n">
@@ -3508,38 +3508,38 @@
         <v>1</v>
       </c>
       <c r="I70" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129112267.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129128838.htm</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Cho thuê nhà nguyên căn</t>
+          <t>Cho thuê phòng HOTEL gần Crowne, FPT, BV 600 giường,...</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>1,3 triệu/tháng</t>
+          <t>3,3 triệu/tháng</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>13 m²</t>
+          <t>32 m²</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F71" t="n">
@@ -3549,31 +3549,31 @@
         <v>0</v>
       </c>
       <c r="H71" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I71" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129125566.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129112267.htm</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>[𝗛𝗔̉𝗜 𝗖𝗛𝗔̂𝗨] 𝗣𝗵𝗼̀𝗻𝗴 𝗙𝘂𝗹𝗹 𝗡𝗼̣̂𝗶 𝗧𝗵𝗮̂́𝘁 𝗠𝗼̛́𝗶</t>
+          <t>Cho thuê nhà nguyên căn</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>3,4 triệu/tháng</t>
+          <t>1,3 triệu/tháng</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>13 m²</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -3583,51 +3583,51 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F72" t="n">
         <v>0</v>
       </c>
       <c r="G72" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H72" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I72" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129122293.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129125566.htm</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>cho thuê nhà mặt tiền trung tâm , ngay nguyễn phước lan</t>
+          <t>[𝗛𝗔̉𝗜 𝗖𝗛𝗔̂𝗨] 𝗣𝗵𝗼̀𝗻𝗴 𝗙𝘂𝗹𝗹 𝗡𝗼̣̂𝗶 𝗧𝗵𝗮̂́𝘁 𝗠𝗼̛́𝗶</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>4 triệu/tháng</t>
+          <t>3,4 triệu/tháng</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F73" t="n">
@@ -3637,36 +3637,36 @@
         <v>1</v>
       </c>
       <c r="H73" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I73" t="n">
         <v>1</v>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129121298.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129122293.htm</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Phòng vip cho thuê giá rẻ</t>
+          <t>cho thuê nhà mặt tiền trung tâm , ngay nguyễn phước lan</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>3 triệu/tháng</t>
+          <t>4 triệu/tháng</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>35 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3678,24 +3678,24 @@
         <v>0</v>
       </c>
       <c r="G74" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H74" t="n">
         <v>0</v>
       </c>
       <c r="I74" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129080805.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129121298.htm</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>cho thuê phòng trọ quận thanh khê</t>
+          <t>Phòng vip cho thuê giá rẻ</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3705,7 +3705,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>35 m²</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -3719,98 +3719,98 @@
         </is>
       </c>
       <c r="F75" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G75" t="n">
         <v>0</v>
       </c>
       <c r="H75" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I75" t="n">
         <v>0</v>
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129096348.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129080805.htm</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Cho thuê phòng diện tích 20m2 trên đường Hoàng Đức Lương, An Hải Bắc</t>
+          <t>cho thuê phòng trọ quận thanh khê</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>3,3 triệu/tháng</t>
+          <t>3 triệu/tháng</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F76" t="n">
         <v>1</v>
       </c>
       <c r="G76" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H76" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I76" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/127435716.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129096348.htm</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Cho thuê căn hộ đầy đủ nội thất gần Đh Fpt, Việt Hàn</t>
+          <t>Cho thuê phòng diện tích 20m2 trên đường Hoàng Đức Lương, An Hải Bắc</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>3 triệu/tháng</t>
+          <t>3,3 triệu/tháng</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F77" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G77" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H77" t="n">
         <v>0</v>
@@ -3820,34 +3820,34 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128764556.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/127435716.htm</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>cho thuê phòng trọ, thanh vinh 900k, 109/116/10 phạm như xương 1,200k</t>
+          <t>Cho thuê căn hộ đầy đủ nội thất gần Đh Fpt, Việt Hàn</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>900000 đ/tháng</t>
+          <t>3 triệu/tháng</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F78" t="n">
@@ -3860,38 +3860,38 @@
         <v>0</v>
       </c>
       <c r="I78" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129088217.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128764556.htm</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CHỈ TỪ 1TR850/THÁNG VỚI CHỖ Ở ĐẦY ĐỦ TIỆN NGHI CHO 1 NGƯỜI</t>
+          <t>cho thuê phòng trọ, thanh vinh 900k, 109/116/10 phạm như xương 1,200k</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>1,85 triệu/tháng</t>
+          <t>900000 đ/tháng</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>10 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F79" t="n">
@@ -3901,41 +3901,41 @@
         <v>0</v>
       </c>
       <c r="H79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129071161.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129088217.htm</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Phòng đầy đủ tiện nghi chỉ vào ở</t>
+          <t>CHỈ TỪ 1TR850/THÁNG VỚI CHỖ Ở ĐẦY ĐỦ TIỆN NGHI CHO 1 NGƯỜI</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>3 triệu/tháng</t>
+          <t>1,85 triệu/tháng</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>10 m²</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Nội thất cao cấp</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F80" t="n">
@@ -3945,41 +3945,41 @@
         <v>0</v>
       </c>
       <c r="H80" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I80" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128711543.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129071161.htm</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Cho thuê 3 phòng trọ Kiệt Nguyễn Xuân Hữu</t>
+          <t>Phòng đầy đủ tiện nghi chỉ vào ở</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2,2 triệu/tháng</t>
+          <t>3 triệu/tháng</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>100 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất cao cấp</t>
         </is>
       </c>
       <c r="F81" t="n">
@@ -3996,24 +3996,24 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129082151.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128711543.htm</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Phòng Trọ Cho Thuê Rộng</t>
+          <t>Cho thuê 3 phòng trọ Kiệt Nguyễn Xuân Hữu</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2,5 triệu/tháng</t>
+          <t>2,2 triệu/tháng</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>35 m²</t>
+          <t>100 m²</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -4023,7 +4023,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F82" t="n">
@@ -4036,38 +4036,38 @@
         <v>0</v>
       </c>
       <c r="I82" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129081900.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129082151.htm</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>🔥Hot! Phòng VIP đối diện bãi biển Nguyễn Tất Thành</t>
+          <t>Phòng Trọ Cho Thuê Rộng</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>7 triệu/tháng</t>
+          <t>2,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>35 m²</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Nội thất cao cấp</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F83" t="n">
@@ -4080,23 +4080,23 @@
         <v>0</v>
       </c>
       <c r="I83" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129077873.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129081900.htm</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>🔥Phòng VIP full nội thất view balcon gần bãi biển Mỹ Khuê</t>
+          <t>🔥Hot! Phòng VIP đối diện bãi biển Nguyễn Tất Thành</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>5,5 triệu/tháng</t>
+          <t>7 triệu/tháng</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -4106,7 +4106,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -4128,14 +4128,14 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129077553.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129077873.htm</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Căn hộ full nội thất Hòa Cường Bắc</t>
+          <t>🔥Phòng VIP full nội thất view balcon gần bãi biển Mỹ Khuê</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -4150,7 +4150,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -4159,7 +4159,7 @@
         </is>
       </c>
       <c r="F85" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G85" t="n">
         <v>0</v>
@@ -4172,19 +4172,19 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128138926.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129077553.htm</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ</t>
+          <t>Căn hộ full nội thất Hòa Cường Bắc</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>3 triệu/tháng</t>
+          <t>5,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -4194,7 +4194,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -4203,7 +4203,7 @@
         </is>
       </c>
       <c r="F86" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G86" t="n">
         <v>0</v>
@@ -4216,34 +4216,34 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129038584.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128138926.htm</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>phòng trọ 43m2,1 tủ có thể kê thêm tiện ích nếu cần</t>
+          <t>Cho thuê phòng trọ</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>3,5 triệu/tháng</t>
+          <t>3 triệu/tháng</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>43 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất cao cấp</t>
         </is>
       </c>
       <c r="F87" t="n">
@@ -4260,34 +4260,34 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129034786.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129038584.htm</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Phòng đầy đủ nội thất thoáng mát CMT8 gần UBND Cẩm Lệ</t>
+          <t>phòng trọ 43m2,1 tủ có thể kê thêm tiện ích nếu cần</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>3 triệu/tháng</t>
+          <t>3,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>22 m²</t>
+          <t>43 m²</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F88" t="n">
@@ -4300,33 +4300,33 @@
         <v>0</v>
       </c>
       <c r="I88" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129057766.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129034786.htm</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Chính chủ cho thuê phòng 1.7tr/ tháng đã bao điện nước tại Cầu Rồng</t>
+          <t>Phòng đầy đủ nội thất thoáng mát CMT8 gần UBND Cẩm Lệ</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>1,7 triệu/tháng</t>
+          <t>3 triệu/tháng</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>22 m²</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -4335,10 +4335,10 @@
         </is>
       </c>
       <c r="F89" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G89" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H89" t="n">
         <v>0</v>
@@ -4348,34 +4348,34 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129043372.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129057766.htm</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Căn hộ 1 phòng ngủ 50m2 - Hải Châu Đà Nẵng</t>
+          <t>Chính chủ cho thuê phòng 1.7tr/ tháng đã bao điện nước tại Cầu Rồng</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>6,5 triệu/tháng</t>
+          <t>1,7 triệu/tháng</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>50 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Nội thất cao cấp</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F90" t="n">
@@ -4388,42 +4388,42 @@
         <v>0</v>
       </c>
       <c r="I90" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128988916.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129043372.htm</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CHO THUÊ CĂN HỘ MỚI GẦN BÃI BIỂN MỸ AN - KHÔNG GIAN YÊN TĨNH</t>
+          <t>Cần nam ở ghép nhà rộng rãi tại đầu đường Tôn Đản, có đầy đủ tiện nghi</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>6,3 triệu/tháng</t>
+          <t>1 triệu/tháng</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>79 m²</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Nội thất cao cấp</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G91" t="n">
         <v>0</v>
@@ -4436,24 +4436,24 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128991832.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128099349.htm</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Cần nam ở ghép nhà rộng rãi tại đầu đường Tôn Đản, có đầy đủ tiện nghi</t>
+          <t>Phòng trọ mới , đường rộng ngây cầu nguyễn tri phương</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>1 triệu/tháng</t>
+          <t>3,6 triệu/tháng</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>79 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F92" t="n">
@@ -4476,23 +4476,23 @@
         <v>0</v>
       </c>
       <c r="I92" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128099349.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129001680.htm</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Phòng trọ mới , đường rộng ngây cầu nguyễn tri phương</t>
+          <t>Phòng Trung Tâm TP</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>3,6 triệu/tháng</t>
+          <t>2,2 triệu/tháng</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -4502,16 +4502,16 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F93" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G93" t="n">
         <v>0</v>
@@ -4520,23 +4520,23 @@
         <v>0</v>
       </c>
       <c r="I93" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129001680.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128935386.htm</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Phòng Trung Tâm TP</t>
+          <t>phòng khách sạn cho thuê tháng đầy đủ tiện nghị</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2,2 triệu/tháng</t>
+          <t>3,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -4546,46 +4546,46 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F94" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G94" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H94" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I94" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128935386.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128858276.htm</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>phòng khách sạn cho thuê tháng đầy đủ tiện nghị</t>
+          <t>Phòng Thoáng Mát Chợ Chiều Mân Thái - Cạnh Biển - Sát Chợ Chiều</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>3,5 triệu/tháng</t>
+          <t>28 triệu/tháng</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>19 m²</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -4595,7 +4595,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F95" t="n">
@@ -4605,31 +4605,31 @@
         <v>1</v>
       </c>
       <c r="H95" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I95" t="n">
         <v>1</v>
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128858276.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128869855.htm</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Phòng Thoáng Mát Chợ Chiều Mân Thái - Cạnh Biển - Sát Chợ Chiều</t>
+          <t>Phòng Mặt Tiền Có Thể Kinh Doanh - K108 Chợ Chiều Mân Thái</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>28 triệu/tháng</t>
+          <t>35 triệu/tháng</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>19 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -4639,7 +4639,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F96" t="n">
@@ -4656,29 +4656,29 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128869855.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128868526.htm</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Phòng Mặt Tiền Có Thể Kinh Doanh - K108 Chợ Chiều Mân Thái</t>
+          <t>Căn hộ dịch vụ mini apartment Hòa Xuân Cẩm Lệ</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>35 triệu/tháng</t>
+          <t>2,7 triệu/tháng</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -4690,7 +4690,7 @@
         <v>1</v>
       </c>
       <c r="G97" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H97" t="n">
         <v>0</v>
@@ -4700,38 +4700,38 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128868526.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/122592431.htm</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Căn hộ dịch vụ mini apartment Hòa Xuân Cẩm Lệ</t>
+          <t>Phòng trọ 20m2</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2,7 triệu/tháng</t>
+          <t>2,2 triệu/tháng</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F98" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G98" t="n">
         <v>0</v>
@@ -4740,38 +4740,38 @@
         <v>0</v>
       </c>
       <c r="I98" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/122592431.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128838248.htm</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Phòng trọ 20m2</t>
+          <t>Tìm ở chung phòng trọ tiểu la, hải châu gần các trường đại học</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2,2 triệu/tháng</t>
+          <t>2,3 triệu/tháng</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F99" t="n">
@@ -4788,19 +4788,19 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128838248.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128828233.htm</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Tìm ở chung phòng trọ tiểu la, hải châu gần các trường đại học</t>
+          <t>Em cần tìm trọ ở khu vực hòa minh thanh khê</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2,3 triệu/tháng</t>
+          <t>2 triệu/tháng</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -4810,12 +4810,12 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F100" t="n">
@@ -4832,19 +4832,19 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128828233.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128778224.htm</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Em cần tìm trọ ở khu vực hòa minh thanh khê</t>
+          <t>Phòng Trọ Cho Thuê - 12/9 Lý Thường Kiệt, Q.Hải Châu, Tp.Đà Nẵng</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2 triệu/tháng</t>
+          <t>2,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -4854,12 +4854,12 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F101" t="n">
@@ -4869,14 +4869,14 @@
         <v>0</v>
       </c>
       <c r="H101" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I101" t="n">
         <v>0</v>
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128778224.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128635892.htm</t>
         </is>
       </c>
     </row>
@@ -6863,115 +6863,115 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Căn hộ studio cầu rồng</t>
+          <t>Cho thuê phòng trọ hòa khánh đà nẵng</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>5,5 triệu/tháng</t>
+          <t>4 triệu/tháng</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>28 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>Nội thất cao cấp</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F147" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G147" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H147" t="n">
         <v>0</v>
       </c>
       <c r="I147" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128082131.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128062696.htm</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ hòa khánh đà nẵng</t>
+          <t>em cần tìm trọ gần đại học đông á ạ, 1 người ở nữ</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>4 triệu/tháng</t>
+          <t>1,8 triệu/tháng</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F148" t="n">
         <v>0</v>
       </c>
       <c r="G148" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H148" t="n">
         <v>0</v>
       </c>
       <c r="I148" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128062696.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128057713.htm</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>em cần tìm trọ gần đại học đông á ạ, 1 người ở nữ</t>
+          <t>Phòng trọ 25m2 gần Bệnh viện Phụ sản - Nhi Đà Nẵng</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>1,8 triệu/tháng</t>
+          <t>1,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F149" t="n">
@@ -6988,95 +6988,7 @@
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128057713.htm</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" t="inlineStr">
-        <is>
-          <t>Phòng trọ 25m2 gần Bệnh viện Phụ sản - Nhi Đà Nẵng</t>
-        </is>
-      </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>1,5 triệu/tháng</t>
-        </is>
-      </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>25 m²</t>
-        </is>
-      </c>
-      <c r="D150" t="inlineStr">
-        <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
-        </is>
-      </c>
-      <c r="E150" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F150" t="n">
-        <v>0</v>
-      </c>
-      <c r="G150" t="n">
-        <v>0</v>
-      </c>
-      <c r="H150" t="n">
-        <v>0</v>
-      </c>
-      <c r="I150" t="n">
-        <v>0</v>
-      </c>
-      <c r="J150" t="inlineStr">
-        <is>
           <t>https://www.nhatot.com/cho-thue-phong-tro/128043795.htm</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="inlineStr">
-        <is>
-          <t>Phòng rẻ nhất Ngũ Hành Sơn</t>
-        </is>
-      </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>3,8 triệu/tháng</t>
-        </is>
-      </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>40 m²</t>
-        </is>
-      </c>
-      <c r="D151" t="inlineStr">
-        <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
-        </is>
-      </c>
-      <c r="E151" t="inlineStr">
-        <is>
-          <t>Nội thất đầy đủ</t>
-        </is>
-      </c>
-      <c r="F151" t="n">
-        <v>1</v>
-      </c>
-      <c r="G151" t="n">
-        <v>1</v>
-      </c>
-      <c r="H151" t="n">
-        <v>1</v>
-      </c>
-      <c r="I151" t="n">
-        <v>1</v>
-      </c>
-      <c r="J151" t="inlineStr">
-        <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128016776.htm</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto scrape + SQL (from Excel) 2025-12-02 17:20:53
</commit_message>
<xml_diff>
--- a/nhatot_phongtro_danang_all.xlsx
+++ b/nhatot_phongtro_danang_all.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J158"/>
+  <dimension ref="A1:J149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -483,31 +483,31 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Căn hộ mini</t>
+          <t>Cho thuê phòng trọ 293/2 Hùng Vương, Đà Nẵng (gần siêu thị Go-Big C)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>3,5 triệu/tháng</t>
+          <t>2,6 triệu/tháng</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>12 m²</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -516,45 +516,45 @@
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129420585.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129441339.htm</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Phòng trọ 25m2, đầy đủ tiện nghi</t>
+          <t>PHÒNG GÁC LỬNG BÁCH KHOA - SƯ PHẠM - MẸ NHU - FPT - CÓ CỬA SỔ</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2,5 triệu/tháng</t>
+          <t>3,2 triệu/tháng</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>15 m²</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F3" t="n">
         <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -564,73 +564,73 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129419558.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129438412.htm</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Phòng mặt tiền tiện nghi,đầy đủ thiết bị Nguyễn Duy Trinh</t>
+          <t>Phòng trọ mặt tiền</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>3 triệu/tháng</t>
+          <t>4 triệu/tháng</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>15 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/127566741.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129404564.htm</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ, phù hợp với gia đình nhỏ, hoặc người đi làm</t>
+          <t>cho thuê phòng mặt tiền 17/5 Trịnh Hoài Đức</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1,7 triệu/tháng</t>
+          <t>3,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>38 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -639,86 +639,86 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129417134.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129400301.htm</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Nhà trọ 50 Trần Quý Khoách, Phường Hòa Khánh, Đà Nẵng</t>
+          <t>Cho thuê phòng trọ 235/2 Hà Huy Tập</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>3 triệu/tháng</t>
+          <t>2,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>22 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129416342.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129432635.htm</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ gần cầu Rồng, bệnh viện Sơn Trà</t>
+          <t>Cho thuê phòng trọ, phù hợp với gia đình nhỏ, hoặc người đi làm</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>1,5 triệu/tháng</t>
+          <t>1,7 triệu/tháng</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>15 m²</t>
+          <t>38 m²</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -740,29 +740,29 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129414200.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129417134.htm</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Phòng trọ Hải Châu, trung tâm, gần cầu rồng</t>
+          <t>Cho thuê căn hộ tại Ngũ Hành Sơn, làng đại học fptt</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1,5 triệu/tháng</t>
+          <t>3 triệu/tháng</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12 m²</t>
+          <t>24 m²</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -771,27 +771,27 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129393857.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129400495.htm</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PHÒNG SLEEP BOX TRUNG TÂM ĐÀ NẴNG – CHO THUÊ DÀI HẠN</t>
+          <t>Phòng mặt tiền cần cho thuê</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -801,17 +801,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -821,21 +821,21 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129386716.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129428846.htm</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Phòng trọ sát bên trường đại học Kiến Trúc, Đông Á và Ngoại Ngữ</t>
+          <t>Căn hộ mini</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -845,12 +845,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>22.5 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -872,29 +872,29 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129411772.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129420585.htm</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Còn 1 phòng 30m2 giá 3,5tr/tháng đường Sơn Thủy Đông 3</t>
+          <t>Phòng trọ 25m2, đầy đủ tiện nghi</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>3,5 triệu/tháng</t>
+          <t>2,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -903,10 +903,10 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
@@ -916,24 +916,24 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128814012.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129419558.htm</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Cho thuê phòng mới xây xong full nội thất</t>
+          <t>Phòng mặt tiền tiện nghi,đầy đủ thiết bị Nguyễn Duy Trinh</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2,7 triệu/tháng</t>
+          <t>3 triệu/tháng</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>24 m²</t>
+          <t>15 m²</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -943,14 +943,14 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F12" t="n">
         <v>1</v>
       </c>
       <c r="G12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H12" t="n">
         <v>1</v>
@@ -960,78 +960,78 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129406962.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/127566741.htm</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Cần nam ở ghép nhà rộng rãi tại đầu đường Tôn Đản, có đầy đủ tiện nghi</t>
+          <t>Nhà trọ 50 Trần Quý Khoách, Phường Hòa Khánh, Đà Nẵng</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1 triệu/tháng</t>
+          <t>3 triệu/tháng</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>79 m²</t>
+          <t>22 m²</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F13" t="n">
         <v>1</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128099349.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129416342.htm</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Phòng trọ mặt tiền</t>
+          <t>Cho thuê phòng trọ gần cầu Rồng, bệnh viện Sơn Trà</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>4 triệu/tháng</t>
+          <t>1,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>15 m²</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F14" t="n">
@@ -1048,73 +1048,73 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129404564.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129414200.htm</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Chính chủ cho thuê phòng 1.7tr/ tháng đã bao điện nước tại Cầu Rồng</t>
+          <t>Phòng trọ Hải Châu, trung tâm, gần cầu rồng</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1,7 triệu/tháng</t>
+          <t>1,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>12 m²</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129043372.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129393857.htm</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Cho thuê phòng gần bến xe , FPT, sư phạm , duy tân , bách khoa</t>
+          <t>PHÒNG SLEEP BOX TRUNG TÂM ĐÀ NẴNG – CHO THUÊ DÀI HẠN</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>1,4 triệu/tháng</t>
+          <t>1,7 triệu/tháng</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>18 m²</t>
+          <t>10 m²</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1129,41 +1129,41 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128382768.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129386716.htm</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Cho thuê phòng ở 3 đến 4 người . Gia đình</t>
+          <t>Phòng trọ sát bên trường đại học Kiến Trúc, Đông Á và Ngoại Ngữ</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1,8 triệu/tháng</t>
+          <t>3,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>35 m²</t>
+          <t>22.5 m²</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F17" t="n">
@@ -1180,24 +1180,24 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129402910.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129411772.htm</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Mình có phòng giá thuê 1tr2 ,bạn nào đi làm ở liên hệ</t>
+          <t>Còn 1 phòng 30m2 giá 3,5tr/tháng đường Sơn Thủy Đông 3</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>1,2 triệu/tháng</t>
+          <t>3,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>40 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1207,36 +1207,36 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F18" t="n">
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H18" t="n">
         <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129401259.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128814012.htm</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Cho thuê căn hộ tại Ngũ Hành Sơn, làng đại học fptt</t>
+          <t>Cho thuê phòng mới xây xong full nội thất</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>3 triệu/tháng</t>
+          <t>2,7 triệu/tháng</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1251,41 +1251,41 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F19" t="n">
         <v>1</v>
       </c>
       <c r="G19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I19" t="n">
         <v>1</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129400495.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129406962.htm</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>cho thuê phòng mặt tiền 17/5 Trịnh Hoài Đức</t>
+          <t>Cần nam ở ghép nhà rộng rãi tại đầu đường Tôn Đản, có đầy đủ tiện nghi</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>3,5 triệu/tháng</t>
+          <t>1 triệu/tháng</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>79 m²</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1305,85 +1305,85 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I20" t="n">
         <v>0</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129400301.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128099349.htm</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>pass trọ gấp</t>
+          <t>Chính chủ cho thuê phòng 1.7tr/ tháng đã bao điện nước tại Cầu Rồng</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2,7 triệu/tháng</t>
+          <t>1,7 triệu/tháng</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F21" t="n">
         <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H21" t="n">
         <v>0</v>
       </c>
       <c r="I21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129397932.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129043372.htm</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Nhà ở dư phòng cho 2 nữ SV ở chung chủ đường Trần Tống.</t>
+          <t>Cho thuê phòng gần bến xe , FPT, sư phạm , duy tân , bách khoa</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>4 triệu/tháng</t>
+          <t>1,4 triệu/tháng</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>18 m²</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Nội thất cao cấp</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F22" t="n">
@@ -1396,28 +1396,28 @@
         <v>0</v>
       </c>
       <c r="I22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129397766.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128382768.htm</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>cho thuê căn hộ</t>
+          <t>Mình có phòng giá thuê 1tr2 ,phòng ghép (bạn đi làm ở liên hệ)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>3,5 triệu/tháng</t>
+          <t>1,2 triệu/tháng</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>38 m²</t>
+          <t>40 m²</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1427,41 +1427,41 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F23" t="n">
         <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H23" t="n">
         <v>0</v>
       </c>
       <c r="I23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129397182.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129401259.htm</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Phòng trọ 640 Trưng Nữ Vương cho thuê</t>
+          <t>pass trọ gấp</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2 triệu/tháng</t>
+          <t>2,7 triệu/tháng</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>15 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1475,7 +1475,7 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G24" t="n">
         <v>0</v>
@@ -1488,34 +1488,34 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129395740.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129397932.htm</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Phòng trọ gần trường bách khoa, Cao Đẳng kh</t>
+          <t>Nhà ở dư phòng cho 2 nữ SV ở chung chủ đường Trần Tống.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>1 triệu/tháng</t>
+          <t>4 triệu/tháng</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>12 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất cao cấp</t>
         </is>
       </c>
       <c r="F25" t="n">
@@ -1525,80 +1525,80 @@
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129394964.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129397766.htm</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Phòng trọ 16m2 đường Mai Lão Bạng, Q. Hải Châu, Đà Nẵng</t>
+          <t>cho thuê căn hộ</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2,4 triệu/tháng</t>
+          <t>3,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>16 m²</t>
+          <t>38 m²</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F26" t="n">
         <v>0</v>
       </c>
       <c r="G26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I26" t="n">
         <v>1</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128723130.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129397182.htm</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>cho thuê phòng trọ đường Diên Hồng</t>
+          <t>Phòng trọ 640 Trưng Nữ Vương cho thuê</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>3,5 triệu/tháng</t>
+          <t>2 triệu/tháng</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>28 m²</t>
+          <t>15 m²</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1620,34 +1620,34 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129381752.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129395740.htm</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>( chính chủ) CHO THUÊ PHÒNG TRỌ ĐƯỜNG 5M Bắc Đẩu</t>
+          <t>Phòng trọ 16m2 đường Mai Lão Bạng, Q. Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2,8 triệu/tháng</t>
+          <t>2,4 triệu/tháng</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>16 m²</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F28" t="n">
@@ -1657,36 +1657,36 @@
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129389367.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128723130.htm</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>( Chính chủ) CHO THUÊ PHÒNG TRỌ MẶT TIỀN ĐƯỜNG 5M BẮC ĐẨU</t>
+          <t>cho thuê phòng trọ đường Diên Hồng</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2,7 triệu/tháng</t>
+          <t>3,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>28 m²</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1708,34 +1708,34 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129389151.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129381752.htm</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>phòng trọ Ngũ Hành Sơn đối diện chợ Bắc Mỹ An, gần Đại học Kinh tế</t>
+          <t>( chính chủ) CHO THUÊ PHÒNG TRỌ ĐƯỜNG 5M Bắc Đẩu</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>3,2 triệu/tháng</t>
+          <t>2,8 triệu/tháng</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>18 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F30" t="n">
@@ -1745,26 +1745,26 @@
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I30" t="n">
         <v>0</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129280652.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129389367.htm</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Phòng trọ 20m2 đường Nguyễn Phước Nguyên</t>
+          <t>( Chính chủ) CHO THUÊ PHÒNG TRỌ MẶT TIỀN ĐƯỜNG 5M BẮC ĐẨU</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2 triệu/tháng</t>
+          <t>2,7 triệu/tháng</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F31" t="n">
@@ -1789,41 +1789,41 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I31" t="n">
         <v>0</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129379829.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129389151.htm</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CHO THUÊ STUDIO – FULL NỘI THẤT – TẢN ĐÀ, THANH KHÊ</t>
+          <t>phòng trọ Ngũ Hành Sơn đối diện chợ Bắc Mỹ An, gần Đại học Kinh tế</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>6,5 triệu/tháng</t>
+          <t>3,2 triệu/tháng</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>40 m²</t>
+          <t>18 m²</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F32" t="n">
@@ -1833,48 +1833,48 @@
         <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I32" t="n">
         <v>0</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129377798.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129280652.htm</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Cho Thuê Phòng Trọ Full NT, Đ. Lâm Quang Thự, ngay Kinh Dương Vương</t>
+          <t>CHO THUÊ STUDIO – FULL NỘI THẤT – TẢN ĐÀ, THANH KHÊ</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>3,6 triệu/tháng</t>
+          <t>6,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>40 m²</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H33" t="n">
         <v>0</v>
@@ -1884,41 +1884,41 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129344615.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129377798.htm</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>cho thuê phòng trọ</t>
+          <t>Cho Thuê Phòng Trọ Full NT, Đ. Lâm Quang Thự, ngay Kinh Dương Vương</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2,2 triệu/tháng</t>
+          <t>3,6 triệu/tháng</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>16 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H34" t="n">
         <v>0</v>
@@ -1928,38 +1928,38 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129354389.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129344615.htm</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>TRỌ MỚI GẦN BÁCH KHOA,SƯ PHẠM</t>
+          <t>cho thuê phòng trọ</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2,8 triệu/tháng</t>
+          <t>2,2 triệu/tháng</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>16 m²</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Nội thất cao cấp</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G35" t="n">
         <v>0</v>
@@ -1968,28 +1968,28 @@
         <v>0</v>
       </c>
       <c r="I35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129346778.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129354389.htm</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Phòng trọ gần trường Đại học Sư Phạm Đà Nẵng</t>
+          <t>TRỌ MỚI GẦN BÁCH KHOA,SƯ PHẠM</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>1 triệu/tháng</t>
+          <t>2,8 triệu/tháng</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>15 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1999,11 +1999,11 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất cao cấp</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G36" t="n">
         <v>0</v>
@@ -2016,7 +2016,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129368650.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129346778.htm</t>
         </is>
       </c>
     </row>
@@ -3744,7 +3744,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>3,5 triệu/tháng</t>
+          <t>3 triệu/tháng</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -4575,17 +4575,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Phòng sạch mới ken- wc riêng - tắm riêng</t>
+          <t>CHO THUÊ PHÒNG TRONG NHÀ NGUYÊN CĂN</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>1,8 triệu/tháng</t>
+          <t>1,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>21 m²</t>
+          <t>10 m²</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -4595,7 +4595,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F95" t="n">
@@ -4612,29 +4612,29 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129120249.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129141283.htm</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Căn hộ 1 , 2 PN khu vực Mỹ Khê - full nội thất</t>
+          <t>Phòng trọ mới , đường rộng ngây cầu nguyễn tri phương</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>13 triệu/tháng</t>
+          <t>3,6 triệu/tháng</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>55 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -4652,33 +4652,33 @@
         <v>0</v>
       </c>
       <c r="I96" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129132617.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129001680.htm</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Cho thuê trọ gác lửng bạn công</t>
+          <t>Phòng Trung Tâm TP</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2,5 triệu/tháng</t>
+          <t>2,2 triệu/tháng</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>22 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -4696,89 +4696,89 @@
         <v>0</v>
       </c>
       <c r="I97" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129123911.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128935386.htm</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CHO THUÊ PHÒNG TRONG NHÀ NGUYÊN CĂN</t>
+          <t>phòng khách sạn cho thuê tháng đầy đủ tiện nghị</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>1,5 triệu/tháng</t>
+          <t>3,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>10 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F98" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G98" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H98" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I98" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129141283.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128858276.htm</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CHO THUÊ PHÒNG TRỌ NGAY PHỐ ĐI BỘ ĐƯỜNG AN THƯỢNG 2</t>
+          <t>Phòng Thoáng Mát Chợ Chiều Mân Thái - Cạnh Biển - Sát Chợ Chiều</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2,5 triệu/tháng</t>
+          <t>28 triệu/tháng</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>16 m²</t>
+          <t>19 m²</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F99" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G99" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H99" t="n">
         <v>0</v>
@@ -4788,68 +4788,68 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129137717.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128869855.htm</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Phòng trọ 21m2 đường Bùi Chát- quận Liên Chiểu</t>
+          <t>Phòng Mặt Tiền Có Thể Kinh Doanh - K108 Chợ Chiều Mân Thái</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>1,6 triệu/tháng</t>
+          <t>35 triệu/tháng</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>21 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F100" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G100" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H100" t="n">
         <v>0</v>
       </c>
       <c r="I100" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129129385.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128868526.htm</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>MỜI THUE TRỌ</t>
+          <t>Căn hộ dịch vụ mini apartment Hòa Xuân Cẩm Lệ</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2 triệu/tháng</t>
+          <t>3 triệu/tháng</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>15 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -4859,51 +4859,51 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F101" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G101" t="n">
         <v>0</v>
       </c>
       <c r="H101" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I101" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129128838.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/122592431.htm</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Cho thuê nhà nguyên căn</t>
+          <t>Phòng trọ 20m2</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>1,3 triệu/tháng</t>
+          <t>2,2 triệu/tháng</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>13 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F102" t="n">
@@ -4920,24 +4920,24 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129125566.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128838248.htm</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>[𝗛𝗔̉𝗜 𝗖𝗛𝗔̂𝗨] 𝗣𝗵𝗼̀𝗻𝗴 𝗙𝘂𝗹𝗹 𝗡𝗼̣̂𝗶 𝗧𝗵𝗮̂́𝘁 𝗠𝗼̛́𝗶</t>
+          <t>Tìm ở chung phòng trọ tiểu la, hải châu gần các trường đại học</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>3,4 triệu/tháng</t>
+          <t>2,3 triệu/tháng</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -4947,80 +4947,80 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F103" t="n">
         <v>0</v>
       </c>
       <c r="G103" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H103" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I103" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129122293.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128828233.htm</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>cho thuê nhà mặt tiền trung tâm , ngay nguyễn phước lan</t>
+          <t>Em cần tìm trọ ở khu vực hòa minh thanh khê</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>4 triệu/tháng</t>
+          <t>2 triệu/tháng</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F104" t="n">
         <v>0</v>
       </c>
       <c r="G104" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H104" t="n">
         <v>0</v>
       </c>
       <c r="I104" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129121298.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128778224.htm</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Phòng trọ mới , đường rộng ngây cầu nguyễn tri phương</t>
+          <t>Phòng Trọ Cho Thuê - 12/9 Lý Thường Kiệt, Q.Hải Châu, Tp.Đà Nẵng</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>3,6 triệu/tháng</t>
+          <t>2,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -5030,7 +5030,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -5039,37 +5039,37 @@
         </is>
       </c>
       <c r="F105" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G105" t="n">
         <v>0</v>
       </c>
       <c r="H105" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I105" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129001680.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128635892.htm</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Phòng Trung Tâm TP</t>
+          <t>THUÊ PHÒNG TRỌ THEO THÁNG</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2,2 triệu/tháng</t>
+          <t>1,8 triệu/tháng</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -5079,7 +5079,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F106" t="n">
@@ -5096,14 +5096,14 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128935386.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128741538.htm</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>phòng khách sạn cho thuê tháng đầy đủ tiện nghị</t>
+          <t>🌟TRỌ GÁC LỬNG MỚI KHU HÒA HẢI _ NGŨ HÀNH SƠN</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -5113,56 +5113,56 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F107" t="n">
         <v>1</v>
       </c>
       <c r="G107" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H107" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I107" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128858276.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128739411.htm</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Phòng Thoáng Mát Chợ Chiều Mân Thái - Cạnh Biển - Sát Chợ Chiều</t>
+          <t>cần tìm nam ở ghép</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>28 triệu/tháng</t>
+          <t>2,9 triệu/tháng</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>19 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -5171,32 +5171,32 @@
         </is>
       </c>
       <c r="F108" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G108" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H108" t="n">
         <v>0</v>
       </c>
       <c r="I108" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128869855.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128737766.htm</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Phòng Mặt Tiền Có Thể Kinh Doanh - K108 Chợ Chiều Mân Thái</t>
+          <t>Cho thuê phòng trọ 20m2 đường Lê Văn Tâm, Đà Nẵng</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>35 triệu/tháng</t>
+          <t>3 triệu/tháng</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -5206,60 +5206,60 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F109" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G109" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H109" t="n">
         <v>0</v>
       </c>
       <c r="I109" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128868526.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128712780.htm</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Căn hộ dịch vụ mini apartment Hòa Xuân Cẩm Lệ</t>
+          <t>Cho thuê phòng trọ sạch đẹp</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>3 triệu/tháng</t>
+          <t>8 triệu/tháng</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>12 m²</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F110" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G110" t="n">
         <v>0</v>
@@ -5268,45 +5268,45 @@
         <v>0</v>
       </c>
       <c r="I110" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/122592431.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128696892.htm</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Phòng trọ 20m2</t>
+          <t>CHO THUÊ NHÀ NGUYÊN CĂN - Kiệt 142 Điện Biên Phủ, TP Đà Nẵng.</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2,2 triệu/tháng</t>
+          <t>8 triệu/tháng</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>40 m²</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F111" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G111" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H111" t="n">
         <v>0</v>
@@ -5316,34 +5316,34 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128838248.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128664350.htm</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Tìm ở chung phòng trọ tiểu la, hải châu gần các trường đại học</t>
+          <t>phòng trọ giá rẻ</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2,3 triệu/tháng</t>
+          <t>1,2 triệu/tháng</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F112" t="n">
@@ -5353,36 +5353,36 @@
         <v>0</v>
       </c>
       <c r="H112" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I112" t="n">
         <v>0</v>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128828233.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128662301.htm</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Em cần tìm trọ ở khu vực hòa minh thanh khê</t>
+          <t>Cho thuê 2 phòng tại k550/6 điện biên phủ, đà nẵng. kiệt 5m</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2 triệu/tháng</t>
+          <t>4 triệu/tháng</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>15 m²</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -5404,24 +5404,24 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128778224.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128654982.htm</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Phòng Trọ Cho Thuê - 12/9 Lý Thường Kiệt, Q.Hải Châu, Tp.Đà Nẵng</t>
+          <t>CHO THUÊ NGUYÊN TẦNG</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2,5 triệu/tháng</t>
+          <t>6 triệu/tháng</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>70 m²</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -5431,7 +5431,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F114" t="n">
@@ -5441,41 +5441,41 @@
         <v>0</v>
       </c>
       <c r="H114" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I114" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128635892.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128619762.htm</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>THUÊ PHÒNG TRỌ THEO THÁNG</t>
+          <t>Cho thuê phòng trọ (dành cho Nam)</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>1,8 triệu/tháng</t>
+          <t>3,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F115" t="n">
@@ -5488,42 +5488,42 @@
         <v>0</v>
       </c>
       <c r="I115" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128741538.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128612931.htm</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>🌟TRỌ GÁC LỬNG MỚI KHU HÒA HẢI _ NGŨ HÀNH SƠN</t>
+          <t>cho thuê phòng full nội thất cao cấp</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>3,5 triệu/tháng</t>
+          <t>7,9 triệu/tháng</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>50 m²</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất cao cấp</t>
         </is>
       </c>
       <c r="F116" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G116" t="n">
         <v>0</v>
@@ -5536,34 +5536,34 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128739411.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128581505.htm</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>cần tìm nam ở ghép</t>
+          <t>Căn hộ Nguyễn Thị Định cho thuê</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2,9 triệu/tháng</t>
+          <t>6 triệu/tháng</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>35 m²</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F117" t="n">
@@ -5580,24 +5580,24 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128737766.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128555766.htm</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ 20m2 đường Lê Văn Tâm, Đà Nẵng</t>
+          <t>kím bạn nữ ở ghép</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>3 triệu/tháng</t>
+          <t>1,3 triệu/tháng</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -5607,7 +5607,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F118" t="n">
@@ -5624,34 +5624,34 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128712780.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128537507.htm</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ sạch đẹp</t>
+          <t>CHO THUÊ PHÒNG TRỌ NGAY BẾN XE TRUNG TÂM ĐÀ NẴNG</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>8 triệu/tháng</t>
+          <t>3 triệu/tháng</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>12 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F119" t="n">
@@ -5664,45 +5664,45 @@
         <v>0</v>
       </c>
       <c r="I119" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128696892.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128523320.htm</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>CHO THUÊ NHÀ NGUYÊN CĂN - Kiệt 142 Điện Biên Phủ, TP Đà Nẵng.</t>
+          <t>Cho thuê Căn hộ, phòng trọ từ 17 -25m</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>8 triệu/tháng</t>
+          <t>2,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>40 m²</t>
+          <t>17 m²</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F120" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G120" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H120" t="n">
         <v>0</v>
@@ -5712,24 +5712,24 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128664350.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128341602.htm</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>phòng trọ giá rẻ</t>
+          <t>CHO THUÊ CĂN STUDIO - NGŨ HÀNH SƠN</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>1,2 triệu/tháng</t>
+          <t>6,2 triệu/tháng</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>40 m²</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -5739,7 +5739,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F121" t="n">
@@ -5756,78 +5756,78 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128662301.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128488165.htm</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Cho thuê 2 phòng tại k550/6 điện biên phủ, đà nẵng. kiệt 5m</t>
+          <t>PASS CĂN HỘ ĐƯỜNG TRƯƠNG QUANG GIAO-CẨM LỆ THÁNG 11 CÓ THỂ CHUYỂN VÀO</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>4 triệu/tháng</t>
+          <t>4,8 triệu/tháng</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>15 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F122" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G122" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H122" t="n">
         <v>0</v>
       </c>
       <c r="I122" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128654982.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128479841.htm</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>CHO THUÊ NGUYÊN TẦNG</t>
+          <t>Tìm bạn ở ghép ( nam) ở lâu dài càng tốt</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>6 triệu/tháng</t>
+          <t>1,25 triệu/tháng</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>70 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F123" t="n">
@@ -5837,36 +5837,36 @@
         <v>0</v>
       </c>
       <c r="H123" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I123" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128619762.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128470096.htm</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ (dành cho Nam)</t>
+          <t>Phòng trọ yên khê 1</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>3,5 triệu/tháng</t>
+          <t>2,6 triệu/tháng</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -5881,31 +5881,31 @@
         <v>0</v>
       </c>
       <c r="H124" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I124" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128612931.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128456987.htm</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>cho thuê phòng full nội thất cao cấp</t>
+          <t>Cho thuê căn hộ cao cấp giá sinh viên</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>7,9 triệu/tháng</t>
+          <t>5,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>50 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -5932,38 +5932,38 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128581505.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128436792.htm</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Căn hộ Nguyễn Thị Định cho thuê</t>
+          <t>Pass phòng ạ, KĐT FPT, ở được 4 người, cho nuôi pet</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>6 triệu/tháng</t>
+          <t>4,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>35 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nội thất cao cấp</t>
         </is>
       </c>
       <c r="F126" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G126" t="n">
         <v>0</v>
@@ -5976,19 +5976,19 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128555766.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128430121.htm</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>kím bạn nữ ở ghép</t>
+          <t>Cho thuê phòng trọ giá tốt gần ĐH Đông Á, Kiến Trúc</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>1,3 triệu/tháng</t>
+          <t>3,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -5998,12 +5998,12 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F127" t="n">
@@ -6016,82 +6016,82 @@
         <v>0</v>
       </c>
       <c r="I127" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128537507.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128419135.htm</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>CHO THUÊ PHÒNG TRỌ NGAY BẾN XE TRUNG TÂM ĐÀ NẴNG</t>
+          <t>Phòng trọ mới xây Núi Thành ngay quảng trường 2/9 từ 3tr5 đến 4tr2</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>3 triệu/tháng</t>
+          <t>4,2 triệu/tháng</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F128" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G128" t="n">
         <v>0</v>
       </c>
       <c r="H128" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I128" t="n">
         <v>1</v>
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128523320.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128403387.htm</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Cho thuê Căn hộ, phòng trọ từ 17 -25m</t>
+          <t>Em cần tìm trọ khu vực cẩm lệ Đà Nẵng ạ ai có liên hê em liền nha</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2,5 triệu/tháng</t>
+          <t>2 triệu/tháng</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>17 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F129" t="n">
@@ -6108,34 +6108,34 @@
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128341602.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128402676.htm</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>CHO THUÊ CĂN STUDIO - NGŨ HÀNH SƠN</t>
+          <t>CHO THUÊ PHÒNG TRỌ</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>6,2 triệu/tháng</t>
+          <t>2,8 triệu/tháng</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>40 m²</t>
+          <t>24 m²</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F130" t="n">
@@ -6145,173 +6145,173 @@
         <v>0</v>
       </c>
       <c r="H130" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I130" t="n">
         <v>0</v>
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128488165.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128398809.htm</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>PASS CĂN HỘ ĐƯỜNG TRƯƠNG QUANG GIAO-CẨM LỆ THÁNG 11 CÓ THỂ CHUYỂN VÀO</t>
+          <t>Chính chủ cho cho thuê phòng căn hộ</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>4,8 triệu/tháng</t>
+          <t>3,7 triệu/tháng</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>28 m²</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F131" t="n">
         <v>1</v>
       </c>
       <c r="G131" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H131" t="n">
         <v>0</v>
       </c>
       <c r="I131" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128479841.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128310448.htm</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Tìm bạn ở ghép ( nam) ở lâu dài càng tốt</t>
+          <t>Cho thuê căn hộ mini đường Bùi Vịnh, Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>1,25 triệu/tháng</t>
+          <t>3,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>27 m²</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F132" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G132" t="n">
         <v>0</v>
       </c>
       <c r="H132" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I132" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128470096.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128381967.htm</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Phòng trọ yên khê 1</t>
+          <t>3 NAM 2007 TÌM 1 BẠN Ở GHÉP CÁCH ĐHKT 1,2KM</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2,6 triệu/tháng</t>
+          <t>1,6 triệu/tháng</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F133" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G133" t="n">
         <v>0</v>
       </c>
       <c r="H133" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I133" t="n">
         <v>0</v>
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128456987.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128377616.htm</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Cho thuê căn hộ cao cấp giá sinh viên</t>
+          <t>tìm người ở ghép cùng</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>5,5 triệu/tháng</t>
+          <t>1,3 triệu/tháng</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>10 m²</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Nội thất cao cấp</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F134" t="n">
@@ -6328,38 +6328,38 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128436792.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128367431.htm</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Pass phòng ạ, KĐT FPT, ở được 4 người, cho nuôi pet</t>
+          <t>CHO THUÊ NHÀ RIÊNG BIỆT MẶT TIỀN 8M ĐƯỜNG 5m5 ( đối diện trường học )</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>4,5 triệu/tháng</t>
+          <t>6,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>50 m²</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Nội thất cao cấp</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F135" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G135" t="n">
         <v>0</v>
@@ -6372,14 +6372,14 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128430121.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128365157.htm</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ giá tốt gần ĐH Đông Á, Kiến Trúc</t>
+          <t>🌿✨ CHO THUÊ PHÒNG TRỌ / CĂN HỘ ✨🌿</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -6389,17 +6389,17 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>13 m²</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F136" t="n">
@@ -6409,21 +6409,21 @@
         <v>0</v>
       </c>
       <c r="H136" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I136" t="n">
         <v>1</v>
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128419135.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128334166.htm</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Phòng trọ mới xây Núi Thành ngay quảng trường 2/9 từ 3tr5 đến 4tr2</t>
+          <t>CHÍNH CHỦ CHO THUÊ PHÒNG – NGAY TRUNG TÂM ĐÀ NẴNG</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -6438,12 +6438,12 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F137" t="n">
@@ -6453,41 +6453,41 @@
         <v>0</v>
       </c>
       <c r="H137" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I137" t="n">
         <v>1</v>
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128403387.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128269219.htm</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Em cần tìm trọ khu vực cẩm lệ Đà Nẵng ạ ai có liên hê em liền nha</t>
+          <t>Cho thuê toà căn hộ 4 tầng 7 phòng đường Đoàn Khuê</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2 triệu/tháng</t>
+          <t>28 triệu/tháng</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>100 m²</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F138" t="n">
@@ -6504,34 +6504,34 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128402676.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128235142.htm</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>CHO THUÊ PHÒNG TRỌ</t>
+          <t>cho thuê nhà nguyên căn</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2,8 triệu/tháng</t>
+          <t>8,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>24 m²</t>
+          <t>104 m²</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F139" t="n">
@@ -6548,29 +6548,29 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128398809.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128230872.htm</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Chính chủ cho cho thuê phòng căn hộ</t>
+          <t>Cho thuê nhà khu vực quang châu hòa phước</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>3,7 triệu/tháng</t>
+          <t>1,7 triệu/tháng</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>28 m²</t>
+          <t>100 m²</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Huyện Hòa Vang, Đà Nẵng</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
@@ -6579,7 +6579,7 @@
         </is>
       </c>
       <c r="F140" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G140" t="n">
         <v>0</v>
@@ -6592,24 +6592,24 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128310448.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128228939.htm</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Cho thuê căn hộ mini đường Bùi Vịnh, Cẩm Lệ, Đà Nẵng</t>
+          <t>Cần cho thê phòng trọ giá rẻ</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>3,5 triệu/tháng</t>
+          <t>2,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>27 m²</t>
+          <t>40 m²</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -6623,7 +6623,7 @@
         </is>
       </c>
       <c r="F141" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G141" t="n">
         <v>0</v>
@@ -6632,33 +6632,33 @@
         <v>0</v>
       </c>
       <c r="I141" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128381967.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128227046.htm</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>3 NAM 2007 TÌM 1 BẠN Ở GHÉP CÁCH ĐHKT 1,2KM</t>
+          <t>Phòng trọ đường Hà Bổng</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>1,6 triệu/tháng</t>
+          <t>3,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
@@ -6667,10 +6667,10 @@
         </is>
       </c>
       <c r="F142" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G142" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H142" t="n">
         <v>0</v>
@@ -6680,24 +6680,24 @@
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128377616.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128217671.htm</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>tìm người ở ghép cùng</t>
+          <t>GÁC LỬNG Ở ĐƯỢC 3 BẠN - ĐƯỜNG TRẦN NGỌC SƯƠNG - GẦN ĐÔNG Á KIẾN TRÚC</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>1,3 triệu/tháng</t>
+          <t>3,6 triệu/tháng</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>10 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -6707,46 +6707,46 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F143" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G143" t="n">
         <v>0</v>
       </c>
       <c r="H143" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I143" t="n">
         <v>0</v>
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128367431.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128189959.htm</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>CHO THUÊ NHÀ RIÊNG BIỆT MẶT TIỀN 8M ĐƯỜNG 5m5 ( đối diện trường học )</t>
+          <t>Phòng trọ có gác lửng, nhà vệ sinh riêng, gần chợ trường học</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>6,5 triệu/tháng</t>
+          <t>2,3 triệu/tháng</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>50 m²</t>
+          <t>16 m²</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
@@ -6768,34 +6768,34 @@
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128365157.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128184395.htm</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>🌿✨ CHO THUÊ PHÒNG TRỌ / CĂN HỘ ✨🌿</t>
+          <t>Phòng Trọ Ngay Mặt Đường</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>3,5 triệu/tháng</t>
+          <t>4 triệu/tháng</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>13 m²</t>
+          <t>45 m²</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F145" t="n">
@@ -6805,80 +6805,80 @@
         <v>0</v>
       </c>
       <c r="H145" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I145" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128334166.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128177160.htm</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>CHÍNH CHỦ CHO THUÊ PHÒNG – NGAY TRUNG TÂM ĐÀ NẴNG</t>
+          <t>Phòng trọ/ Căn hộ</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>4,2 triệu/tháng</t>
+          <t>5 triệu/tháng</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>35 m²</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F146" t="n">
         <v>1</v>
       </c>
       <c r="G146" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H146" t="n">
         <v>0</v>
       </c>
       <c r="I146" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128269219.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128173132.htm</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Cho thuê toà căn hộ 4 tầng 7 phòng đường Đoàn Khuê</t>
+          <t>Cho thuê 3 phòng 24m2 tầng 2&amp;3</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>28 triệu/tháng</t>
+          <t>3,3 triệu/tháng</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>100 m²</t>
+          <t>24 m²</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
@@ -6887,42 +6887,42 @@
         </is>
       </c>
       <c r="F147" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G147" t="n">
         <v>0</v>
       </c>
       <c r="H147" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I147" t="n">
         <v>0</v>
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128235142.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128172121.htm</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>cho thuê nhà nguyên căn</t>
+          <t>Cho thuê phòng trọ</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>8,5 triệu/tháng</t>
+          <t>2,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>104 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
@@ -6944,29 +6944,29 @@
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128230872.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128159779.htm</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Cho thuê nhà khu vực quang châu hòa phước</t>
+          <t>Cho thuê phòng trọ đường Trần Văn Thành - Ngũ Hành Sơn - Đà Nẵng</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>1,7 triệu/tháng</t>
+          <t>2,4 triệu/tháng</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>100 m²</t>
+          <t>18 m²</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Huyện Hòa Vang, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
@@ -6987,402 +6987,6 @@
         <v>0</v>
       </c>
       <c r="J149" t="inlineStr">
-        <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128228939.htm</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" t="inlineStr">
-        <is>
-          <t>Cần cho thê phòng trọ giá rẻ</t>
-        </is>
-      </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>2,5 triệu/tháng</t>
-        </is>
-      </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>40 m²</t>
-        </is>
-      </c>
-      <c r="D150" t="inlineStr">
-        <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
-        </is>
-      </c>
-      <c r="E150" t="inlineStr">
-        <is>
-          <t>Nội thất đầy đủ</t>
-        </is>
-      </c>
-      <c r="F150" t="n">
-        <v>0</v>
-      </c>
-      <c r="G150" t="n">
-        <v>0</v>
-      </c>
-      <c r="H150" t="n">
-        <v>0</v>
-      </c>
-      <c r="I150" t="n">
-        <v>0</v>
-      </c>
-      <c r="J150" t="inlineStr">
-        <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128227046.htm</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="inlineStr">
-        <is>
-          <t>Phòng trọ đường Hà Bổng</t>
-        </is>
-      </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>3,5 triệu/tháng</t>
-        </is>
-      </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>25 m²</t>
-        </is>
-      </c>
-      <c r="D151" t="inlineStr">
-        <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
-        </is>
-      </c>
-      <c r="E151" t="inlineStr">
-        <is>
-          <t>Nội thất đầy đủ</t>
-        </is>
-      </c>
-      <c r="F151" t="n">
-        <v>0</v>
-      </c>
-      <c r="G151" t="n">
-        <v>1</v>
-      </c>
-      <c r="H151" t="n">
-        <v>0</v>
-      </c>
-      <c r="I151" t="n">
-        <v>0</v>
-      </c>
-      <c r="J151" t="inlineStr">
-        <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128217671.htm</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="inlineStr">
-        <is>
-          <t>GÁC LỬNG Ở ĐƯỢC 3 BẠN - ĐƯỜNG TRẦN NGỌC SƯƠNG - GẦN ĐÔNG Á KIẾN TRÚC</t>
-        </is>
-      </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>3,6 triệu/tháng</t>
-        </is>
-      </c>
-      <c r="C152" t="inlineStr">
-        <is>
-          <t>25 m²</t>
-        </is>
-      </c>
-      <c r="D152" t="inlineStr">
-        <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
-        </is>
-      </c>
-      <c r="E152" t="inlineStr">
-        <is>
-          <t>Nội thất đầy đủ</t>
-        </is>
-      </c>
-      <c r="F152" t="n">
-        <v>1</v>
-      </c>
-      <c r="G152" t="n">
-        <v>0</v>
-      </c>
-      <c r="H152" t="n">
-        <v>1</v>
-      </c>
-      <c r="I152" t="n">
-        <v>0</v>
-      </c>
-      <c r="J152" t="inlineStr">
-        <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128189959.htm</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t>Phòng trọ có gác lửng, nhà vệ sinh riêng, gần chợ trường học</t>
-        </is>
-      </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>2,3 triệu/tháng</t>
-        </is>
-      </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>16 m²</t>
-        </is>
-      </c>
-      <c r="D153" t="inlineStr">
-        <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
-        </is>
-      </c>
-      <c r="E153" t="inlineStr">
-        <is>
-          <t>Nhà trống</t>
-        </is>
-      </c>
-      <c r="F153" t="n">
-        <v>0</v>
-      </c>
-      <c r="G153" t="n">
-        <v>0</v>
-      </c>
-      <c r="H153" t="n">
-        <v>0</v>
-      </c>
-      <c r="I153" t="n">
-        <v>0</v>
-      </c>
-      <c r="J153" t="inlineStr">
-        <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128184395.htm</t>
-        </is>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="inlineStr">
-        <is>
-          <t>Phòng Trọ Ngay Mặt Đường</t>
-        </is>
-      </c>
-      <c r="B154" t="inlineStr">
-        <is>
-          <t>4 triệu/tháng</t>
-        </is>
-      </c>
-      <c r="C154" t="inlineStr">
-        <is>
-          <t>45 m²</t>
-        </is>
-      </c>
-      <c r="D154" t="inlineStr">
-        <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
-        </is>
-      </c>
-      <c r="E154" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F154" t="n">
-        <v>0</v>
-      </c>
-      <c r="G154" t="n">
-        <v>0</v>
-      </c>
-      <c r="H154" t="n">
-        <v>0</v>
-      </c>
-      <c r="I154" t="n">
-        <v>0</v>
-      </c>
-      <c r="J154" t="inlineStr">
-        <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128177160.htm</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="inlineStr">
-        <is>
-          <t>Phòng trọ/ Căn hộ</t>
-        </is>
-      </c>
-      <c r="B155" t="inlineStr">
-        <is>
-          <t>5 triệu/tháng</t>
-        </is>
-      </c>
-      <c r="C155" t="inlineStr">
-        <is>
-          <t>35 m²</t>
-        </is>
-      </c>
-      <c r="D155" t="inlineStr">
-        <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
-        </is>
-      </c>
-      <c r="E155" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F155" t="n">
-        <v>1</v>
-      </c>
-      <c r="G155" t="n">
-        <v>1</v>
-      </c>
-      <c r="H155" t="n">
-        <v>0</v>
-      </c>
-      <c r="I155" t="n">
-        <v>0</v>
-      </c>
-      <c r="J155" t="inlineStr">
-        <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128173132.htm</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" t="inlineStr">
-        <is>
-          <t>Cho thuê 3 phòng 24m2 tầng 2&amp;3</t>
-        </is>
-      </c>
-      <c r="B156" t="inlineStr">
-        <is>
-          <t>3,3 triệu/tháng</t>
-        </is>
-      </c>
-      <c r="C156" t="inlineStr">
-        <is>
-          <t>24 m²</t>
-        </is>
-      </c>
-      <c r="D156" t="inlineStr">
-        <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
-        </is>
-      </c>
-      <c r="E156" t="inlineStr">
-        <is>
-          <t>Nội thất đầy đủ</t>
-        </is>
-      </c>
-      <c r="F156" t="n">
-        <v>1</v>
-      </c>
-      <c r="G156" t="n">
-        <v>0</v>
-      </c>
-      <c r="H156" t="n">
-        <v>1</v>
-      </c>
-      <c r="I156" t="n">
-        <v>0</v>
-      </c>
-      <c r="J156" t="inlineStr">
-        <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128172121.htm</t>
-        </is>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" t="inlineStr">
-        <is>
-          <t>Cho thuê phòng trọ</t>
-        </is>
-      </c>
-      <c r="B157" t="inlineStr">
-        <is>
-          <t>2,5 triệu/tháng</t>
-        </is>
-      </c>
-      <c r="C157" t="inlineStr">
-        <is>
-          <t>30 m²</t>
-        </is>
-      </c>
-      <c r="D157" t="inlineStr">
-        <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
-        </is>
-      </c>
-      <c r="E157" t="inlineStr">
-        <is>
-          <t>Nhà trống</t>
-        </is>
-      </c>
-      <c r="F157" t="n">
-        <v>0</v>
-      </c>
-      <c r="G157" t="n">
-        <v>0</v>
-      </c>
-      <c r="H157" t="n">
-        <v>0</v>
-      </c>
-      <c r="I157" t="n">
-        <v>0</v>
-      </c>
-      <c r="J157" t="inlineStr">
-        <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128159779.htm</t>
-        </is>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" t="inlineStr">
-        <is>
-          <t>Cho thuê phòng trọ đường Trần Văn Thành - Ngũ Hành Sơn - Đà Nẵng</t>
-        </is>
-      </c>
-      <c r="B158" t="inlineStr">
-        <is>
-          <t>2,4 triệu/tháng</t>
-        </is>
-      </c>
-      <c r="C158" t="inlineStr">
-        <is>
-          <t>18 m²</t>
-        </is>
-      </c>
-      <c r="D158" t="inlineStr">
-        <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
-        </is>
-      </c>
-      <c r="E158" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F158" t="n">
-        <v>0</v>
-      </c>
-      <c r="G158" t="n">
-        <v>0</v>
-      </c>
-      <c r="H158" t="n">
-        <v>0</v>
-      </c>
-      <c r="I158" t="n">
-        <v>0</v>
-      </c>
-      <c r="J158" t="inlineStr">
         <is>
           <t>https://www.nhatot.com/cho-thue-phong-tro/128154852.htm</t>
         </is>

</xml_diff>

<commit_message>
Auto scrape + SQL (from Excel) 2026-02-09 17:49:41
</commit_message>
<xml_diff>
--- a/nhatot_phongtro_danang_all.xlsx
+++ b/nhatot_phongtro_danang_all.xlsx
@@ -483,27 +483,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>cho thuê căn hộ studio full nội thất . vị trí gần biển , chợ ,siêu thị</t>
+          <t>cho thue phòng gần Tiểu La - LeThanhNghi</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>4 triệu/tháng</t>
+          <t>2,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>15 m²</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -513,41 +513,41 @@
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129934394.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130489969.htm</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Phòng trọ làng đại học ĐN - li xi năm âm lịch</t>
+          <t>PHÒNG CHO THUÊ CAO CẤP - TRUNG TÂM TP</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2,2 triệu/tháng</t>
+          <t>2,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -557,41 +557,41 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130676812.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129322964.htm</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PHÒNG TRỌ - SLEEP BOX gần cầu Trần Thị Lý , cầu Rồng.</t>
+          <t>Phòng trọ làng đại học ĐN - li xi năm âm lịch</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1,7 triệu/tháng</t>
+          <t>2,2 triệu/tháng</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>10 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -601,36 +601,36 @@
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130171786.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130676812.htm</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TRỐNG PHÒNG MẶT TIỀN SAU LƯNG BẾN XE TP ĐÀ NẴNG VÀO Ở ĐƯỢC NGAY</t>
+          <t>PHÒNG TRỌ - SLEEP BOX gần cầu Trần Thị Lý , cầu Rồng.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2,5 triệu/tháng</t>
+          <t>1,7 triệu/tháng</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>10 m²</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -645,41 +645,41 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130616941.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130171786.htm</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>cho thuê phòng trọ sinh viên/ gia đình nhỏ</t>
+          <t>cho thuê căn hộ studio full nội thất . vị trí gần biển , chợ ,siêu thị</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1,8 triệu/tháng</t>
+          <t>4 triệu/tháng</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>18 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -696,24 +696,24 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130705122.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129934394.htm</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Cho thuê phòng mặt tiền 68/20 Nguyễn mộng tuân ngay bến xe</t>
+          <t>Phòng trọ giá rẻ</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>4 triệu/tháng</t>
+          <t>1,2 triệu/tháng</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -733,31 +733,31 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129217669.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130256253.htm</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Phòng trọ giá rẻ</t>
+          <t>Phòng trọ trống</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1,2 triệu/tháng</t>
+          <t>1,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>15 m²</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -767,7 +767,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F8" t="n">
@@ -784,29 +784,29 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130256253.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130612949.htm</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Phòng diện tích 30m2, Hoà Xuân</t>
+          <t>CĂN HỘ MI NI GIA ĐÌNH GẦN CHỢ HÒA KHÁNH</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>3,8 triệu/tháng</t>
+          <t>2,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -815,10 +815,10 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
@@ -828,19 +828,19 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130390633.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129652506.htm</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Phòng Trọ MT số 147 Nguyễn Quyền cạnh BX Trung Tâm</t>
+          <t>cho thuê trọ</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2,5 triệu/tháng</t>
+          <t>3,2 triệu/tháng</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -850,16 +850,16 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
@@ -872,29 +872,29 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130616972.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130727446.htm</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MẶT TIỀN ĐƯỜNG HOÀNG DIỆU CHO THUÊ PHÒNG ĐẦY ĐỦ TIỆN NGHI</t>
+          <t>cho thuê phòng trọ</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>3,5 triệu/tháng</t>
+          <t>1 triệu/tháng</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>19 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -903,47 +903,47 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130492770.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130726074.htm</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>phòng trọ sát biển đầy đủ nội thất thoáng mát</t>
+          <t>cho thuê phòng trọ kiệt lê hữu trác</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>3,2 triệu/tháng</t>
+          <t>1,6 triệu/tháng</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>16 m²</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -960,29 +960,29 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130706830.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130725829.htm</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>NHÀ TRỌ MỚI CẦN CHO THUÊ TẠI TRUNG TÂM</t>
+          <t>TRỐNG PHÒNG MẶT TIỀN SAU LƯNG BẾN XE TP ĐÀ NẴNG VÀO Ở ĐƯỢC NGAY</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>3 triệu/tháng</t>
+          <t>2,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>60 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -997,26 +997,26 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130692858.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130616941.htm</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>𝑪𝒉𝒐 𝒕𝒉𝒖𝒆̂ 𝒑𝒉𝒐̀𝒏𝒈 𝒕𝒓𝒐̣ 𝒕𝒓𝒖𝒏𝒈 𝒕𝒂̂𝒎 Quận Hải Châu</t>
+          <t>Cho thuê phòng mặt tiền 68/20 Nguyễn mộng tuân ngay bến xe</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>3 triệu/tháng</t>
+          <t>4 triệu/tháng</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1026,63 +1026,63 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130695328.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129217669.htm</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Phòng Trọ Mới Xây có NỘI THẤT gần ĐH Bách Khoa KCN</t>
+          <t>Phòng diện tích 30m2, Hoà Xuân</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2,4 triệu/tháng</t>
+          <t>3,8 triệu/tháng</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F15" t="n">
         <v>1</v>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -1092,29 +1092,29 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129892147.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130390633.htm</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Phòng trọ Hoàng Diệu TTTP</t>
+          <t>Phòng Trọ MT số 147 Nguyễn Quyền cạnh BX Trung Tâm</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2,8 triệu/tháng</t>
+          <t>2,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1126,34 +1126,34 @@
         <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130092935.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130616972.htm</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ 38 m2 đường 10,5m Trịnh công Sơn</t>
+          <t>MẶT TIỀN ĐƯỜNG HOÀNG DIỆU CHO THUÊ PHÒNG ĐẦY ĐỦ TIỆN NGHI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>4,5 triệu/tháng</t>
+          <t>3,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>38 m²</t>
+          <t>19 m²</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1163,46 +1163,46 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130694895.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130492770.htm</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Cho Thuê Phòng ngay TTTP ngày 15/02 trống, Đ. Lý Thường Kiệt</t>
+          <t>phòng trọ sát biển đầy đủ nội thất thoáng mát</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>3,3 triệu/tháng</t>
+          <t>3,2 triệu/tháng</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1211,10 +1211,10 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H18" t="n">
         <v>0</v>
@@ -1224,41 +1224,41 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130678522.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130706830.htm</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>cho thuê phòng đầy đủ tiện nghi tại 4/3 lưu quang thuận, mỹ an, ĐN</t>
+          <t>NHÀ TRỌ MỚI CẦN CHO THUÊ TẠI TRUNG TÂM</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>3,2 triệu/tháng</t>
+          <t>3 triệu/tháng</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>22 m²</t>
+          <t>60 m²</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H19" t="n">
         <v>1</v>
@@ -1268,19 +1268,19 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130677326.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130692858.htm</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Đang…TRỐNG… 01 phòng mặt tiền cho ai cần ( Chuyển vào ngay )</t>
+          <t>𝑪𝒉𝒐 𝒕𝒉𝒖𝒆̂ 𝒑𝒉𝒐̀𝒏𝒈 𝒕𝒓𝒐̣ 𝒕𝒓𝒖𝒏𝒈 𝒕𝒂̂𝒎 Quận Hải Châu</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>3,8 triệu/tháng</t>
+          <t>3 triệu/tháng</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1290,7 +1290,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1299,47 +1299,47 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130678353.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130695328.htm</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>cho thuê phòng trọ 63 đường hoàng đình ái</t>
+          <t>Phòng Trọ Mới Xây có NỘI THẤT gần ĐH Bách Khoa KCN</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>3 triệu/tháng</t>
+          <t>2,4 triệu/tháng</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F21" t="n">
@@ -1349,31 +1349,31 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130667204.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129892147.htm</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CHỈ TỪ 1TR850/THÁNG VỚI CHỖ Ở ĐẦY ĐỦ TIỆN NGHI CHO 1 NGƯỜI</t>
+          <t>Phòng trọ Hoàng Diệu TTTP</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>1,85 triệu/tháng</t>
+          <t>2,8 triệu/tháng</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>10 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1383,46 +1383,46 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F22" t="n">
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I22" t="n">
         <v>1</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129071161.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130092935.htm</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Trống 1 căn hộ full nội thất đường Nguyễn Xiển - Ngũ Hành Sơn</t>
+          <t>Cho thuê phòng trọ 38 m2 đường 10,5m Trịnh công Sơn</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>3,5 triệu/tháng</t>
+          <t>4,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>35 m²</t>
+          <t>38 m²</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1431,7 +1431,7 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G23" t="n">
         <v>0</v>
@@ -1440,23 +1440,23 @@
         <v>0</v>
       </c>
       <c r="I23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130684528.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130694895.htm</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Phòng trọ 3 sao mới xây tiện nghi Nguyễn Duy Trinh</t>
+          <t>Cho Thuê Phòng ngay TTTP ngày 15/02 trống, Đ. Lý Thường Kiệt</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2,2 triệu/tháng</t>
+          <t>3,3 triệu/tháng</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1466,12 +1466,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F24" t="n">
@@ -1481,85 +1481,85 @@
         <v>1</v>
       </c>
       <c r="H24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130683785.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130678522.htm</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ mới, sạch, đẹp – Dọn vào ở ngay</t>
+          <t>cho thuê phòng đầy đủ tiện nghi tại 4/3 lưu quang thuận, mỹ an, ĐN</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>3 triệu/tháng</t>
+          <t>3,2 triệu/tháng</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>15 m²</t>
+          <t>22 m²</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I25" t="n">
         <v>1</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130683511.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130677326.htm</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ khu vực KCN Hoà Cầm giá rẻ</t>
+          <t>Đang…TRỐNG… 01 phòng mặt tiền cho ai cần ( Chuyển vào ngay )</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>700000 đ/tháng</t>
+          <t>3,8 triệu/tháng</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>10 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F26" t="n">
@@ -1576,29 +1576,29 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130626785.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130678353.htm</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CHO THUÊ PHÒNG STUDIO FULL NỘI THẤT – SƠN TRÀ, ĐÀ NẴNG</t>
+          <t>cho thuê phòng trọ 63 đường hoàng đình ái</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>8 triệu/tháng</t>
+          <t>3 triệu/tháng</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>40 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1607,37 +1607,37 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130677977.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130667204.htm</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Phòng trọ đường Hoàng Diệu, điều hoà nội thất đầy đủ, giờ giấc tự do</t>
+          <t>CHỈ TỪ 1TR850/THÁNG VỚI CHỖ Ở ĐẦY ĐỦ TIỆN NGHI CHO 1 NGƯỜI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2,5 triệu/tháng</t>
+          <t>1,85 triệu/tháng</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>10 m²</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1660,42 +1660,42 @@
         <v>1</v>
       </c>
       <c r="I28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130663007.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129071161.htm</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Cho thuê phòng gần bến xe , FPT, sư phạm , duy tân , bách khoa</t>
+          <t>Trống 1 căn hộ full nội thất đường Nguyễn Xiển - Ngũ Hành Sơn</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>1,6 triệu/tháng</t>
+          <t>3,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>35 m²</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G29" t="n">
         <v>0</v>
@@ -1704,28 +1704,28 @@
         <v>0</v>
       </c>
       <c r="I29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128382768.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130684528.htm</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>PHÒNG TRỌ ĐẦY ĐỦ NỘI THẤT, MỚI, KV  FPT, ĐH VIỆT HÀN, NON NƯỚC</t>
+          <t>Phòng trọ 3 sao mới xây tiện nghi Nguyễn Duy Trinh</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2,9 triệu/tháng</t>
+          <t>2,2 triệu/tháng</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>17 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F30" t="n">
@@ -1745,41 +1745,41 @@
         <v>1</v>
       </c>
       <c r="H30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I30" t="n">
         <v>1</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130644644.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130683785.htm</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Phòng xinh xắn - Bình yên bên biển</t>
+          <t>Cho thuê phòng trọ mới, sạch, đẹp – Dọn vào ở ngay</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>5 triệu/tháng</t>
+          <t>3 triệu/tháng</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>15 m²</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F31" t="n">
@@ -1789,48 +1789,48 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130669995.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130683511.htm</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Trọ dorm sleepbox đủ hết tiện nghi-Hoà Cường Bắc-Bao điện nước</t>
+          <t>Cho thuê phòng trọ khu vực KCN Hoà Cầm giá rẻ</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>1,4 triệu/tháng</t>
+          <t>700000 đ/tháng</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>10 m²</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H32" t="n">
         <v>0</v>
@@ -1840,34 +1840,34 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129917316.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130626785.htm</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Phòng trọ full nội thất gần trường Kinh tế</t>
+          <t>CHO THUÊ PHÒNG STUDIO FULL NỘI THẤT – SƠN TRÀ, ĐÀ NẴNG</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>3,2 triệu/tháng</t>
+          <t>8 triệu/tháng</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>40 m²</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F33" t="n">
@@ -1877,26 +1877,26 @@
         <v>1</v>
       </c>
       <c r="H33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130664916.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130677977.htm</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CHO THUÊ PHÒNG TRỌ GÁC LỬNG MỚI XÂY</t>
+          <t>Phòng trọ đường Hoàng Diệu, điều hoà nội thất đầy đủ, giờ giấc tự do</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>3,3 triệu/tháng</t>
+          <t>2,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1915,51 +1915,51 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G34" t="n">
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130659080.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130663007.htm</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Phòng Căn Hộ Đầy Đủ Nội Thất</t>
+          <t>Cho thuê phòng gần bến xe , FPT, sư phạm , duy tân , bách khoa</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>4 triệu/tháng</t>
+          <t>1,6 triệu/tháng</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>24 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G35" t="n">
         <v>0</v>
@@ -1972,24 +1972,24 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130632574.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128382768.htm</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Cho thuê phòng full nội thất, rộng rãi , có ban công . Gần ĐH Fpt</t>
+          <t>PHÒNG TRỌ ĐẦY ĐỦ NỘI THẤT, MỚI, KV  FPT, ĐH VIỆT HÀN, NON NƯỚC</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>4,2 triệu/tháng</t>
+          <t>2,9 triệu/tháng</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>45 m²</t>
+          <t>17 m²</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2003,10 +2003,10 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H36" t="n">
         <v>0</v>
@@ -2016,19 +2016,19 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130652083.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130644644.htm</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Cho thuê phòng giường tầng phòng dorm</t>
+          <t>Phòng xinh xắn - Bình yên bên biển</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>1 triệu/tháng</t>
+          <t>5 triệu/tháng</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2038,7 +2038,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2050,39 +2050,39 @@
         <v>0</v>
       </c>
       <c r="G37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128128560.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130669995.htm</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>🏡 𝗞𝗵𝗮𝗶 𝗧𝗿𝘂̛𝗼̛𝗻𝗴 𝗣𝗵𝗼̀𝗻𝗴 𝗙𝘂𝗹𝗹 𝗡𝗼̣̂𝗶 𝗧𝗵𝗮̂́𝘁 𝗠𝗼̛́𝗶 𝟭𝟬𝟬% - 𝗼̛̉ 𝗧𝗿𝘂𝗻𝗴 𝗧𝗮̂𝗺</t>
+          <t>Phòng trọ full nội thất gần trường Kinh tế</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>4,6 triệu/tháng</t>
+          <t>3,2 triệu/tháng</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>35 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2091,7 +2091,7 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G38" t="n">
         <v>1</v>
@@ -2100,33 +2100,33 @@
         <v>1</v>
       </c>
       <c r="I38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130645343.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130664916.htm</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>cho thuê căn full nội thất</t>
+          <t>Phòng Căn Hộ Đầy Đủ Nội Thất</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>5 triệu/tháng</t>
+          <t>4 triệu/tháng</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>35 m²</t>
+          <t>24 m²</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2135,7 +2135,7 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G39" t="n">
         <v>0</v>
@@ -2148,34 +2148,34 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130644830.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130632574.htm</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Cho thuê căn hộ Sơn Trà</t>
+          <t>Cho thuê phòng full nội thất, rộng rãi , có ban công . Gần ĐH Fpt</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>10 triệu/tháng</t>
+          <t>4,2 triệu/tháng</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>100 m²</t>
+          <t>45 m²</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F40" t="n">
@@ -2188,33 +2188,33 @@
         <v>0</v>
       </c>
       <c r="I40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130643512.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130652083.htm</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Phòng trọ có gác Hàm Nghi gần ĐH Duy Tân, Khu trung tâm Ng. Văn Linh</t>
+          <t>Cho thuê phòng giường tầng phòng dorm</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2,9 triệu/tháng</t>
+          <t>1 triệu/tháng</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>15 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2223,91 +2223,91 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H41" t="n">
         <v>0</v>
       </c>
       <c r="I41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130616960.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128128560.htm</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Nguyễn Như Hạnh-Hòa Minh-Liên Chiểu</t>
+          <t>🏡 𝗞𝗵𝗮𝗶 𝗧𝗿𝘂̛𝗼̛𝗻𝗴 𝗣𝗵𝗼̀𝗻𝗴 𝗙𝘂𝗹𝗹 𝗡𝗼̣̂𝗶 𝗧𝗵𝗮̂́𝘁 𝗠𝗼̛́𝗶 𝟭𝟬𝟬% - 𝗼̛̉ 𝗧𝗿𝘂𝗻𝗴 𝗧𝗮̂𝗺</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>4 triệu/tháng</t>
+          <t>4,6 triệu/tháng</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>18 m²</t>
+          <t>35 m²</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130615408.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130645343.htm</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ đẹp mini</t>
+          <t>cho thuê căn full nội thất</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2,8 triệu/tháng</t>
+          <t>5 triệu/tháng</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>22 m²</t>
+          <t>35 m²</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Nội thất cao cấp</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F43" t="n">
@@ -2317,41 +2317,41 @@
         <v>0</v>
       </c>
       <c r="H43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I43" t="n">
         <v>0</v>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130603781.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130644830.htm</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Phòng trọ mặt tiền</t>
+          <t>Cho thuê căn hộ Sơn Trà</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2,5 triệu/tháng</t>
+          <t>10 triệu/tháng</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>100 m²</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F44" t="n">
@@ -2368,24 +2368,24 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130639136.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130643512.htm</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>(Tháng 2) Chính chủ Cho thuê dãy nhà trọ mặt tiền đường Trần Can</t>
+          <t>Phòng trọ có gác Hàm Nghi gần ĐH Duy Tân, Khu trung tâm Ng. Văn Linh</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2 triệu/tháng</t>
+          <t>2,9 triệu/tháng</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>15 m²</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -2399,7 +2399,7 @@
         </is>
       </c>
       <c r="F45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G45" t="n">
         <v>0</v>
@@ -2412,29 +2412,29 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128261428.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130616960.htm</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ gần bãi tắm mỹ khê, bv 199, chợ phước mỹ 2tr5</t>
+          <t>Nguyễn Như Hạnh-Hòa Minh-Liên Chiểu</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2,5 triệu/tháng</t>
+          <t>4 triệu/tháng</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>18 m²</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2456,34 +2456,34 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130626864.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130615408.htm</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Nhà cho thuê có gát lửng</t>
+          <t>Cho thuê phòng trọ đẹp mini</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2,7 triệu/tháng</t>
+          <t>2,8 triệu/tháng</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>15 m²</t>
+          <t>22 m²</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất cao cấp</t>
         </is>
       </c>
       <c r="F47" t="n">
@@ -2493,21 +2493,21 @@
         <v>0</v>
       </c>
       <c r="H47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I47" t="n">
         <v>0</v>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130626676.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130603781.htm</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Trọ 35m2 Tại Hải Châu 19 Nguyễn Thành Ý, Gần Đại Học Đông Á, Kiến Trúc</t>
+          <t>Phòng trọ mặt tiền</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2517,12 +2517,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>35 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2544,29 +2544,29 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130301716.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130639136.htm</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Trọ 2tr8 Tiểu La, trung tâm</t>
+          <t>(Tháng 2) Chính chủ Cho thuê dãy nhà trọ mặt tiền đường Trần Can</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2,8 triệu/tháng</t>
+          <t>2 triệu/tháng</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>15 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2588,34 +2588,34 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130623413.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128261428.htm</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ 20m2 số 49 Đường Liêm Lạc 18, Hòa Xuân, Đà Nẵng</t>
+          <t>Cho thuê phòng trọ gần bãi tắm mỹ khê, bv 199, chợ phước mỹ 2tr5</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>1,5 triệu/tháng</t>
+          <t>2,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F50" t="n">
@@ -2632,14 +2632,14 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130619420.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130626864.htm</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Căn hộ dịch vụ mini apartment Hòa Xuân Cẩm Lệ</t>
+          <t>Nhà cho thuê có gát lửng</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2649,21 +2649,21 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>15 m²</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G51" t="n">
         <v>0</v>
@@ -2672,33 +2672,33 @@
         <v>0</v>
       </c>
       <c r="I51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/122592431.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130626676.htm</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Phòng trọ trống</t>
+          <t>Trọ 35m2 Tại Hải Châu 19 Nguyễn Thành Ý, Gần Đại Học Đông Á, Kiến Trúc</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>1,5 triệu/tháng</t>
+          <t>2,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>15 m²</t>
+          <t>35 m²</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2713,41 +2713,41 @@
         <v>0</v>
       </c>
       <c r="H52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I52" t="n">
         <v>0</v>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130612949.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130301716.htm</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Phòng trọ 20m2 đường Trần Cao Vân, Q. Thanh Khê</t>
+          <t>Trọ 2tr8 Tiểu La, trung tâm</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2 triệu/tháng</t>
+          <t>2,8 triệu/tháng</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>15 m²</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F53" t="n">
@@ -2764,19 +2764,19 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130610077.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130623413.htm</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Cho thuê phòng đầy đủ tiện nghi</t>
+          <t>Cho thuê phòng trọ 20m2 số 49 Đường Liêm Lạc 18, Hòa Xuân, Đà Nẵng</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>3,4 triệu/tháng</t>
+          <t>1,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2786,60 +2786,60 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F54" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G54" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H54" t="n">
         <v>0</v>
       </c>
       <c r="I54" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130588824.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130619420.htm</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Cho thuê trọ</t>
+          <t>Căn hộ dịch vụ mini apartment Hòa Xuân Cẩm Lệ</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>1,6 triệu/tháng</t>
+          <t>2,7 triệu/tháng</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G55" t="n">
         <v>0</v>
@@ -2848,23 +2848,23 @@
         <v>0</v>
       </c>
       <c r="I55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130605821.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/122592431.htm</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Cho thuê phòng khu vip Thi Sách</t>
+          <t>Phòng trọ 20m2 đường Trần Cao Vân, Q. Thanh Khê</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2,7 triệu/tháng</t>
+          <t>2 triệu/tháng</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2874,7 +2874,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2896,19 +2896,19 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130604471.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130610077.htm</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CHO THUÊ PHÒNG TRỌ MỚI ĐẦY ĐỦ NỘI THẤT Ở KHU LÀNG ĐẠI HỌC NGŨ HÀNH SƠN</t>
+          <t>Cho thuê phòng đầy đủ tiện nghi</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>3,2 triệu/tháng</t>
+          <t>3,4 triệu/tháng</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2930,29 +2930,29 @@
         <v>1</v>
       </c>
       <c r="G57" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H57" t="n">
         <v>0</v>
       </c>
       <c r="I57" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130525716.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130588824.htm</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CHO THUÊ PHÒNG MỚI ĐẦY ĐỦ NỘI THẤT SÁT ĐH VIỆT HÀN  VÀ FPT</t>
+          <t>Cho thuê trọ</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>3 triệu/tháng</t>
+          <t>1,6 triệu/tháng</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2967,36 +2967,36 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F58" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G58" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H58" t="n">
         <v>0</v>
       </c>
       <c r="I58" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130587817.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130605821.htm</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Phòng trọ Trung Tâm - Cao Thắng &amp; Đống Đa</t>
+          <t>Cho thuê phòng khu vip Thi Sách</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>1 triệu/tháng</t>
+          <t>2,7 triệu/tháng</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -3028,29 +3028,29 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130578598.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130604471.htm</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Có phòng trọ cho thuê dọn vào ở ngay, sát sông hàn</t>
+          <t>CHO THUÊ PHÒNG TRỌ MỚI ĐẦY ĐỦ NỘI THẤT Ở KHU LÀNG ĐẠI HỌC NGŨ HÀNH SƠN</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2,8 triệu/tháng</t>
+          <t>3,2 triệu/tháng</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -3059,76 +3059,76 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G60" t="n">
         <v>0</v>
       </c>
       <c r="H60" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I60" t="n">
         <v>0</v>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128927575.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130525716.htm</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Phòng trọ</t>
+          <t>CHO THUÊ PHÒNG MỚI ĐẦY ĐỦ NỘI THẤT SÁT ĐH VIỆT HÀN  VÀ FPT</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>1,8 triệu/tháng</t>
+          <t>3 triệu/tháng</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Huyện Hòa Vang, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F61" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G61" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H61" t="n">
         <v>0</v>
       </c>
       <c r="I61" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130577688.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130587817.htm</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>phòng 20 m  cách mặt tiền lê duẩn 20 m</t>
+          <t>Phòng trọ Trung Tâm - Cao Thắng &amp; Đống Đa</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>3,5 triệu/tháng</t>
+          <t>1 triệu/tháng</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -3138,12 +3138,12 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F62" t="n">
@@ -3160,34 +3160,34 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130240755.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130578598.htm</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CHO THUÊ NHÀ 2 PHÒNG NGỦ HÒA XUÂN</t>
+          <t>Có phòng trọ cho thuê dọn vào ở ngay, sát sông hàn</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>7 triệu/tháng</t>
+          <t>2,8 triệu/tháng</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>100 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F63" t="n">
@@ -3197,41 +3197,41 @@
         <v>0</v>
       </c>
       <c r="H63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I63" t="n">
         <v>0</v>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130535874.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128927575.htm</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CĂN ĐẦY ĐỦ NỘI THẤT , CÁCH 5 PHÚT ĐẾN ĐH BÁCH KHOA , KCN HOÀ KHÁNH</t>
+          <t>Phòng trọ</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>1,9 triệu/tháng</t>
+          <t>1,8 triệu/tháng</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>18 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Huyện Hòa Vang, Đà Nẵng</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F64" t="n">
@@ -3241,41 +3241,41 @@
         <v>0</v>
       </c>
       <c r="H64" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130563578.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130577688.htm</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>PHÒNG SLEEP BOX TRUNG TÂM ĐÀ NẴNG – CHO THUÊ DÀI HẠN</t>
+          <t>phòng 20 m  cách mặt tiền lê duẩn 20 m</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>1,7 triệu/tháng</t>
+          <t>3,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>10 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F65" t="n">
@@ -3285,45 +3285,45 @@
         <v>0</v>
       </c>
       <c r="H65" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I65" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129386716.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130240755.htm</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>PHÒNG SLEEPBOX 1.7tr gần CẦU RỒNG, CẦU TRẦN THỊ LÝ đã bao điện nước</t>
+          <t>CHO THUÊ NHÀ 2 PHÒNG NGỦ HÒA XUÂN</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>1,7 triệu/tháng</t>
+          <t>7 triệu/tháng</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>100 m²</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F66" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G66" t="n">
         <v>0</v>
@@ -3336,34 +3336,34 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130549005.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130535874.htm</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ gác lửng tại 158 Trần Đình Nam</t>
+          <t>CĂN ĐẦY ĐỦ NỘI THẤT , CÁCH 5 PHÚT ĐẾN ĐH BÁCH KHOA , KCN HOÀ KHÁNH</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2,5 triệu/tháng</t>
+          <t>1,9 triệu/tháng</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>18 m²</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F67" t="n">
@@ -3373,80 +3373,80 @@
         <v>0</v>
       </c>
       <c r="H67" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I67" t="n">
         <v>0</v>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130547373.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130563578.htm</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Phòng trọ mới xây xong - 2 tầng - giá tốt chỉ 2tr5</t>
+          <t>Cho thuê phòng khu vực sơn trà đà nẵng.</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2,5 triệu/tháng</t>
+          <t>3,3 triệu/tháng</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>28 m²</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G68" t="n">
         <v>0</v>
       </c>
       <c r="H68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I68" t="n">
         <v>0</v>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130545001.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130558442.htm</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CHO THUÊ CĂN HỘ TẠI THANH KHÊ, ĐẦY ĐỦ TIỆN NGHI</t>
+          <t>PHÒNG SLEEP BOX TRUNG TÂM ĐÀ NẴNG – CHO THUÊ DÀI HẠN</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>4 triệu/tháng</t>
+          <t>1,7 triệu/tháng</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>32 m²</t>
+          <t>10 m²</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -3455,10 +3455,10 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G69" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H69" t="n">
         <v>1</v>
@@ -3468,38 +3468,38 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129913117.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129386716.htm</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>phong trọ Nguyen Xuan huu Cam Lệ</t>
+          <t>PHÒNG SLEEPBOX 1.7tr gần CẦU RỒNG, CẦU TRẦN THỊ LÝ đã bao điện nước</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2,4 triệu/tháng</t>
+          <t>1,7 triệu/tháng</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Sơn Trà, Đà Nẵng</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Nội thất cao cấp</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F70" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G70" t="n">
         <v>0</v>
@@ -3512,29 +3512,29 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130502097.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130549005.htm</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Căn hộ phòng khách sạn – Hoàng Diệu, Hải Châu</t>
+          <t>Cho thuê phòng trọ gác lửng tại 158 Trần Đình Nam</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>3,5 triệu/tháng</t>
+          <t>2,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -3556,34 +3556,34 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130191297.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130547373.htm</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>phòng mẹ suốt có gác ngay sau lưng dh sư phạm</t>
+          <t>Phòng trọ mới xây xong - 2 tầng - giá tốt chỉ 2tr5</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>1,5 triệu/tháng</t>
+          <t>2,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>15 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F72" t="n">
@@ -3600,41 +3600,41 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129619654.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130545001.htm</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>PASS PHÒNG GIÁ SINH VIÊN 3 TRIỆU – GẦN ĐH KINH TẾ</t>
+          <t>CHO THUÊ CĂN HỘ TẠI THANH KHÊ, ĐẦY ĐỦ TIỆN NGHI</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>3 triệu/tháng</t>
+          <t>4 triệu/tháng</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>32 m²</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F73" t="n">
         <v>1</v>
       </c>
       <c r="G73" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H73" t="n">
         <v>1</v>
@@ -3644,78 +3644,78 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130522758.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129913117.htm</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Cho thuê phòng trọ gần bến xe trung tâm</t>
+          <t>phong trọ Nguyen Xuan huu Cam Lệ</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2 triệu/tháng</t>
+          <t>2,4 triệu/tháng</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>16 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nội thất cao cấp</t>
         </is>
       </c>
       <c r="F74" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G74" t="n">
         <v>0</v>
       </c>
       <c r="H74" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I74" t="n">
         <v>0</v>
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130517612.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130502097.htm</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CHO THUÊ PHÒNG TRỌ GẦN ĐH SƯ PHẠM, BÁCH KHOA GIÁ RẺ</t>
+          <t>Căn hộ phòng khách sạn – Hoàng Diệu, Hải Châu</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>3 triệu/tháng</t>
+          <t>3,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F75" t="n">
@@ -3728,28 +3728,28 @@
         <v>0</v>
       </c>
       <c r="I75" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130495073.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130191297.htm</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Phòng trọ giá rẻ hòa khánh bắc</t>
+          <t>phòng mẹ suốt có gác ngay sau lưng dh sư phạm</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>1 triệu/tháng</t>
+          <t>1,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>15 m²</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -3759,7 +3759,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F76" t="n">
@@ -3776,68 +3776,68 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130506808.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129619654.htm</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Cho thuê phòng ngay trung tâm thành phố, đầy đủ nội thất, gần trường</t>
+          <t>PASS PHÒNG GIÁ SINH VIÊN 3 TRIỆU – GẦN ĐH KINH TẾ</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>4 triệu/tháng</t>
+          <t>3 triệu/tháng</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F77" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G77" t="n">
         <v>0</v>
       </c>
       <c r="H77" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I77" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130505022.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130522758.htm</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Cho thuê phòng sạch sẽ, an ninh tốt 17/6 Nguyễn Huy Tưởng, Hoà Khánh</t>
+          <t>Cho thuê phòng trọ gần bến xe trung tâm</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2,8 triệu/tháng</t>
+          <t>2 triệu/tháng</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>16 m²</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -3854,7 +3854,7 @@
         <v>1</v>
       </c>
       <c r="G78" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H78" t="n">
         <v>1</v>
@@ -3864,34 +3864,34 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130485834.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130517612.htm</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Cho thuê phòng sạch sẽ, thoáng mát, cửa sổ rộng view trời</t>
+          <t>CHO THUÊ PHÒNG TRỌ GẦN ĐH SƯ PHẠM, BÁCH KHOA GIÁ RẺ</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2,1 triệu/tháng</t>
+          <t>3 triệu/tháng</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>22 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F79" t="n">
@@ -3901,41 +3901,41 @@
         <v>0</v>
       </c>
       <c r="H79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130191204.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130495073.htm</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Phòng 12m2 An Hải Bắc, Sơn Trà Đà Nẵng</t>
+          <t>Phòng trọ giá rẻ hòa khánh bắc</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>1,6 triệu/tháng</t>
+          <t>1 triệu/tháng</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>12 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F80" t="n">
@@ -3952,34 +3952,34 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129284531.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130506808.htm</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Còn trống 1 phòng sạch đẹp-gác lửng (Nguyễn Như Hạnh)</t>
+          <t>Cho thuê phòng ngay trung tâm thành phố, đầy đủ nội thất, gần trường</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2 triệu/tháng</t>
+          <t>4 triệu/tháng</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>18 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F81" t="n">
@@ -3989,41 +3989,41 @@
         <v>0</v>
       </c>
       <c r="H81" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I81" t="n">
         <v>0</v>
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130359756.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130505022.htm</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>PHÒNG GIƯỜNG TẦNG RIÊNG TƯ GẦN ĐH KINH TẾ</t>
+          <t>Cho thuê phòng sạch sẽ, an ninh tốt 17/6 Nguyễn Huy Tưởng, Hoà Khánh</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>950000 đ/tháng</t>
+          <t>2,8 triệu/tháng</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>50 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F82" t="n">
@@ -4033,45 +4033,45 @@
         <v>1</v>
       </c>
       <c r="H82" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I82" t="n">
         <v>0</v>
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130491610.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130485834.htm</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Phòng ban công full nội thất new 100% khu FPT - Ngũ Hành Sơn</t>
+          <t>Cho thuê phòng sạch sẽ, thoáng mát, cửa sổ rộng view trời</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>4 triệu/tháng</t>
+          <t>2,1 triệu/tháng</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>40 m²</t>
+          <t>22 m²</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F83" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G83" t="n">
         <v>0</v>
@@ -4080,72 +4080,72 @@
         <v>1</v>
       </c>
       <c r="I83" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128629777.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130191204.htm</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Phòng Full Nội Thất Khu FPT - Ngũ Hành Sơn</t>
+          <t>Còn trống 1 phòng sạch đẹp-gác lửng (Nguyễn Như Hạnh)</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>3,8 triệu/tháng</t>
+          <t>2 triệu/tháng</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>38 m²</t>
+          <t>18 m²</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F84" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G84" t="n">
         <v>0</v>
       </c>
       <c r="H84" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I84" t="n">
         <v>0</v>
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/128025078.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130359756.htm</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>PHÒNG GÁC LỬNG MỚI - GẦN ĐẠI HỌC FPT - NGŨ HÀNH SƠN</t>
+          <t>PHÒNG GIƯỜNG TẦNG RIÊNG TƯ GẦN ĐH KINH TẾ</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>3,2 triệu/tháng</t>
+          <t>950000 đ/tháng</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>25 m²</t>
+          <t>50 m²</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -4162,48 +4162,48 @@
         <v>1</v>
       </c>
       <c r="G85" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H85" t="n">
         <v>0</v>
       </c>
       <c r="I85" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130490358.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130491610.htm</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Đầu tháng 3 trống phòng gần Tiểu La - LeThanhNghi</t>
+          <t>Phòng ban công full nội thất new 100% khu FPT - Ngũ Hành Sơn</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2,5 triệu/tháng</t>
+          <t>4 triệu/tháng</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>15 m²</t>
+          <t>40 m²</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F86" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G86" t="n">
         <v>0</v>
@@ -4212,42 +4212,42 @@
         <v>1</v>
       </c>
       <c r="I86" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130489969.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128629777.htm</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Phòng trọ 22m2 đường Phạm Nhữ Tăng, Thanh Khê</t>
+          <t>Phòng Full Nội Thất Khu FPT - Ngũ Hành Sơn</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2 triệu/tháng</t>
+          <t>3,8 triệu/tháng</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>22 m²</t>
+          <t>38 m²</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F87" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G87" t="n">
         <v>0</v>
@@ -4260,19 +4260,19 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130489019.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/128025078.htm</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Cần cho thuê phòng trọ, khu TĐC Hòa Liên 4</t>
+          <t>PHÒNG GÁC LỬNG MỚI - GẦN ĐẠI HỌC FPT - NGŨ HÀNH SƠN</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>1,7 triệu/tháng</t>
+          <t>3,2 triệu/tháng</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -4282,16 +4282,16 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Huyện Hòa Vang, Đà Nẵng</t>
+          <t>Quận Ngũ Hành Sơn, Đà Nẵng</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F88" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G88" t="n">
         <v>0</v>
@@ -4300,116 +4300,116 @@
         <v>0</v>
       </c>
       <c r="I88" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130484790.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130490358.htm</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Phòng cho gia đình mini văn hóa</t>
+          <t>Phòng trọ 22m2 đường Phạm Nhữ Tăng, Thanh Khê</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>3,1 triệu/tháng</t>
+          <t>2 triệu/tháng</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>35 m²</t>
+          <t>22 m²</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Quận Sơn Trà, Đà Nẵng</t>
+          <t>Quận Thanh Khê, Đà Nẵng</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F89" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G89" t="n">
         <v>0</v>
       </c>
       <c r="H89" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I89" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130483805.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130489019.htm</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Mình còn trống 1 phòng</t>
+          <t>Cần cho thuê phòng trọ, khu TĐC Hòa Liên 4</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>3,8 triệu/tháng</t>
+          <t>1,7 triệu/tháng</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>25 m²</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Quận Liên Chiểu, Đà Nẵng</t>
+          <t>Huyện Hòa Vang, Đà Nẵng</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Nội thất cao cấp</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F90" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G90" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H90" t="n">
         <v>0</v>
       </c>
       <c r="I90" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130471801.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130484790.htm</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Tôi cần bán phòng trọ kiệt K120 .  Bên hông ĐH bách khoa</t>
+          <t>Mình còn trống 1 phòng</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>3 tỷ/tháng</t>
+          <t>3,8 triệu/tháng</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>100 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -4419,41 +4419,41 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất cao cấp</t>
         </is>
       </c>
       <c r="F91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H91" t="n">
         <v>0</v>
       </c>
       <c r="I91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/129870417.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130471801.htm</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Nhà còn trống 01 phòng trọ, cần cho thuê</t>
+          <t>Tôi cần bán phòng trọ kiệt K120 .  Bên hông ĐH bách khoa</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2,4 triệu/tháng</t>
+          <t>3 tỷ/tháng</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>22 m²</t>
+          <t>100 m²</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F92" t="n">
@@ -4476,42 +4476,42 @@
         <v>0</v>
       </c>
       <c r="I92" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130454910.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/129870417.htm</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>STUDIO "XỊN MỊN" 40m2 NGAY NGUYỄN VĂN LINH - HẢI CHÂU, ĐÀ NẴNG</t>
+          <t>Nhà còn trống 01 phòng trọ, cần cho thuê</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>7 triệu/tháng</t>
+          <t>2,4 triệu/tháng</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>40 m²</t>
+          <t>22 m²</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Quận Hải Châu, Đà Nẵng</t>
+          <t>Quận Liên Chiểu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Nội thất đầy đủ</t>
+          <t>Nhà trống</t>
         </is>
       </c>
       <c r="F93" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G93" t="n">
         <v>0</v>
@@ -4524,38 +4524,38 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130430158.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130454910.htm</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Phòng trọ 30m2 đường Nhơn Hoà 22, Hoà An, Cẩm Lệ, Đà Nẵng</t>
+          <t>STUDIO "XỊN MỊN" 40m2 NGAY NGUYỄN VĂN LINH - HẢI CHÂU, ĐÀ NẴNG</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2,5 triệu/tháng</t>
+          <t>7 triệu/tháng</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>30 m²</t>
+          <t>40 m²</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Quận Cẩm Lệ, Đà Nẵng</t>
+          <t>Quận Hải Châu, Đà Nẵng</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Nội thất đầy đủ</t>
         </is>
       </c>
       <c r="F94" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G94" t="n">
         <v>0</v>
@@ -4564,38 +4564,38 @@
         <v>0</v>
       </c>
       <c r="I94" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130431043.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130430158.htm</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>phòng trọ 12m2 nằm trong hẻm - yêu cầu nữ</t>
+          <t>Phòng trọ 30m2 đường Nhơn Hoà 22, Hoà An, Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>1 triệu/tháng</t>
+          <t>2,5 triệu/tháng</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>12 m²</t>
+          <t>30 m²</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Quận Thanh Khê, Đà Nẵng</t>
+          <t>Quận Cẩm Lệ, Đà Nẵng</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Nhà trống</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F95" t="n">
@@ -4612,7 +4612,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>https://www.nhatot.com/cho-thue-phong-tro/130426624.htm</t>
+          <t>https://www.nhatot.com/cho-thue-phong-tro/130431043.htm</t>
         </is>
       </c>
     </row>

</xml_diff>